<commit_message>
Spieltag 4 (2026/27): Daten, Kaderseiten und Portal-Tabelle aktualisiert
- Datendateien aus D:\Spreeliga\stand aufgefrischt: saison.xlsx, players-se.csv,
  spieltagspunkte.csv, clientdb.json, historie/manager.json, stats/saison.json,
  neu stats/st4.json, stats/powerverlauf.json.
- Alle 11 manager-*.html und portal.html erstmals mit werkstatt\bauen\website.js
  erzeugt statt von Hand umgestellt: Aufstellung Spieltag 4, Formation, Topspieler,
  Gesamtpunkte, Rang aus rangSaison.
- Dabei die Rangfarben vereinheitlicht (Gold/Silber/Bronze fuer 1-3, sonst Grau):
  die Punktekachel war bei Rang 1-3 verrutscht und trug bei Rang 4 und 11 Gold.
- vergleich.html und spieler.html unveraendert (Quellcode seit ST3 gleich).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/saison.xlsx
+++ b/saison.xlsx
@@ -474,6 +474,12 @@
       <c r="J2" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K2">
+        <v>6</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -506,6 +512,12 @@
       <c r="J3" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K3">
+        <v>4</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -538,6 +550,12 @@
       <c r="J4" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K4">
+        <v>-2</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -570,6 +588,12 @@
       <c r="J5" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -602,6 +626,12 @@
       <c r="J6" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K6">
+        <v>2</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -634,6 +664,12 @@
       <c r="J7" t="str">
         <v>Bank</v>
       </c>
+      <c r="K7">
+        <v>2</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -666,6 +702,12 @@
       <c r="J8" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K8">
+        <v>4</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -698,6 +740,12 @@
       <c r="J9" t="str">
         <v>Bank</v>
       </c>
+      <c r="K9">
+        <v>12</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -730,6 +778,12 @@
       <c r="J10" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K10">
+        <v>30</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -762,6 +816,12 @@
       <c r="J11" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K11">
+        <v>13</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -794,6 +854,12 @@
       <c r="J12" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K12">
+        <v>7</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -826,6 +892,12 @@
       <c r="J13" t="str">
         <v>Bank</v>
       </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -858,6 +930,12 @@
       <c r="J14" t="str">
         <v>Bank</v>
       </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -890,6 +968,12 @@
       <c r="J15" t="str">
         <v>Bank</v>
       </c>
+      <c r="K15">
+        <v>2</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -922,6 +1006,12 @@
       <c r="J16" t="str">
         <v>Bank</v>
       </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -954,6 +1044,12 @@
       <c r="J17" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K17">
+        <v>12</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -986,6 +1082,12 @@
       <c r="J18" t="str">
         <v>Bank</v>
       </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1018,6 +1120,12 @@
       <c r="J19" t="str">
         <v>Bank</v>
       </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1050,6 +1158,12 @@
       <c r="J20" t="str">
         <v>Bank</v>
       </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1082,6 +1196,12 @@
       <c r="J21" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1114,6 +1234,12 @@
       <c r="J22" t="str">
         <v>Bank</v>
       </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1146,6 +1272,12 @@
       <c r="J23" t="str">
         <v>Bank</v>
       </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1178,6 +1310,12 @@
       <c r="J24" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K24">
+        <v>8</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1210,6 +1348,12 @@
       <c r="J25" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K25">
+        <v>2</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1236,6 +1380,12 @@
       <c r="H26" t="str">
         <v>Bank</v>
       </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1268,6 +1418,12 @@
       <c r="J27" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1300,6 +1456,12 @@
       <c r="J28" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K28">
+        <v>4</v>
+      </c>
+      <c r="L28" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1332,6 +1494,12 @@
       <c r="J29" t="str">
         <v>Bank</v>
       </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1364,6 +1532,12 @@
       <c r="J30" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K30">
+        <v>8</v>
+      </c>
+      <c r="L30" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1396,6 +1570,12 @@
       <c r="J31" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K31">
+        <v>-2</v>
+      </c>
+      <c r="L31" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1428,6 +1608,12 @@
       <c r="J32" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K32">
+        <v>30</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1460,6 +1646,12 @@
       <c r="J33" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K33">
+        <v>16</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1492,6 +1684,12 @@
       <c r="J34" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K34">
+        <v>13</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1524,6 +1722,12 @@
       <c r="J35" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K35">
+        <v>0</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1556,6 +1760,12 @@
       <c r="J36" t="str">
         <v>Bank</v>
       </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1588,6 +1798,12 @@
       <c r="J37" t="str">
         <v>Bank</v>
       </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -1620,6 +1836,12 @@
       <c r="J38" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1652,6 +1874,12 @@
       <c r="J39" t="str">
         <v>Bank</v>
       </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+      <c r="L39" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1684,6 +1912,12 @@
       <c r="J40" t="str">
         <v>Bank</v>
       </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
+      <c r="L40" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1716,6 +1950,12 @@
       <c r="J41" t="str">
         <v>Bank</v>
       </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -1748,6 +1988,12 @@
       <c r="J42" t="str">
         <v>Bank</v>
       </c>
+      <c r="K42">
+        <v>0</v>
+      </c>
+      <c r="L42" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -1774,6 +2020,12 @@
       <c r="H43" t="str">
         <v>Bank</v>
       </c>
+      <c r="K43">
+        <v>0</v>
+      </c>
+      <c r="L43" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -1806,6 +2058,12 @@
       <c r="J44" t="str">
         <v>Bank</v>
       </c>
+      <c r="K44">
+        <v>0</v>
+      </c>
+      <c r="L44" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -1838,6 +2096,12 @@
       <c r="J45" t="str">
         <v>Bank</v>
       </c>
+      <c r="K45">
+        <v>0</v>
+      </c>
+      <c r="L45" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -1870,6 +2134,12 @@
       <c r="J46" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K46">
+        <v>12</v>
+      </c>
+      <c r="L46" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -1902,6 +2172,12 @@
       <c r="J47" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K47">
+        <v>2</v>
+      </c>
+      <c r="L47" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -1934,6 +2210,12 @@
       <c r="J48" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K48">
+        <v>-2</v>
+      </c>
+      <c r="L48" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -1966,6 +2248,12 @@
       <c r="J49" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K49">
+        <v>-2</v>
+      </c>
+      <c r="L49" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -1998,6 +2286,12 @@
       <c r="J50" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K50">
+        <v>4</v>
+      </c>
+      <c r="L50" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -2030,6 +2324,12 @@
       <c r="J51" t="str">
         <v>Bank</v>
       </c>
+      <c r="K51">
+        <v>0</v>
+      </c>
+      <c r="L51" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -2062,6 +2362,12 @@
       <c r="J52" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K52">
+        <v>0</v>
+      </c>
+      <c r="L52" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -2094,6 +2400,12 @@
       <c r="J53" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K53">
+        <v>2</v>
+      </c>
+      <c r="L53" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -2126,6 +2438,12 @@
       <c r="J54" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K54">
+        <v>30</v>
+      </c>
+      <c r="L54" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -2158,6 +2476,12 @@
       <c r="J55" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K55">
+        <v>7</v>
+      </c>
+      <c r="L55" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2190,6 +2514,12 @@
       <c r="J56" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K56">
+        <v>0</v>
+      </c>
+      <c r="L56" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2222,6 +2552,12 @@
       <c r="J57" t="str">
         <v>Bank</v>
       </c>
+      <c r="K57">
+        <v>0</v>
+      </c>
+      <c r="L57" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -2254,6 +2590,12 @@
       <c r="J58" t="str">
         <v>Bank</v>
       </c>
+      <c r="K58">
+        <v>0</v>
+      </c>
+      <c r="L58" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2286,6 +2628,12 @@
       <c r="J59" t="str">
         <v>Bank</v>
       </c>
+      <c r="K59">
+        <v>0</v>
+      </c>
+      <c r="L59" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -2318,6 +2666,12 @@
       <c r="J60" t="str">
         <v>Bank</v>
       </c>
+      <c r="K60">
+        <v>2</v>
+      </c>
+      <c r="L60" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -2350,6 +2704,12 @@
       <c r="J61" t="str">
         <v>Bank</v>
       </c>
+      <c r="K61">
+        <v>0</v>
+      </c>
+      <c r="L61" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -2382,6 +2742,12 @@
       <c r="J62" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K62">
+        <v>12</v>
+      </c>
+      <c r="L62" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -2414,6 +2780,12 @@
       <c r="J63" t="str">
         <v>Bank</v>
       </c>
+      <c r="K63">
+        <v>0</v>
+      </c>
+      <c r="L63" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -2446,6 +2818,12 @@
       <c r="J64" t="str">
         <v>Bank</v>
       </c>
+      <c r="K64">
+        <v>0</v>
+      </c>
+      <c r="L64" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -2478,6 +2856,12 @@
       <c r="J65" t="str">
         <v>Bank</v>
       </c>
+      <c r="K65">
+        <v>2</v>
+      </c>
+      <c r="L65" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -2510,6 +2894,12 @@
       <c r="J66" t="str">
         <v>Bank</v>
       </c>
+      <c r="K66">
+        <v>-2</v>
+      </c>
+      <c r="L66" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -2542,6 +2932,12 @@
       <c r="J67" t="str">
         <v>Bank</v>
       </c>
+      <c r="K67">
+        <v>0</v>
+      </c>
+      <c r="L67" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -2574,6 +2970,12 @@
       <c r="J68" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K68">
+        <v>8</v>
+      </c>
+      <c r="L68" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -2606,6 +3008,12 @@
       <c r="J69" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K69">
+        <v>0</v>
+      </c>
+      <c r="L69" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -2638,6 +3046,12 @@
       <c r="J70" t="str">
         <v>Bank</v>
       </c>
+      <c r="K70">
+        <v>-2</v>
+      </c>
+      <c r="L70" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -2670,6 +3084,12 @@
       <c r="J71" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K71">
+        <v>2</v>
+      </c>
+      <c r="L71" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2702,6 +3122,12 @@
       <c r="J72" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K72">
+        <v>4</v>
+      </c>
+      <c r="L72" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -2734,6 +3160,12 @@
       <c r="J73" t="str">
         <v>Bank</v>
       </c>
+      <c r="K73">
+        <v>12</v>
+      </c>
+      <c r="L73" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -2766,6 +3198,12 @@
       <c r="J74" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K74">
+        <v>2</v>
+      </c>
+      <c r="L74" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -2798,6 +3236,12 @@
       <c r="J75" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K75">
+        <v>2</v>
+      </c>
+      <c r="L75" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -2830,6 +3274,12 @@
       <c r="J76" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K76">
+        <v>7</v>
+      </c>
+      <c r="L76" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -2862,6 +3312,12 @@
       <c r="J77" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K77">
+        <v>6</v>
+      </c>
+      <c r="L77" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -2894,6 +3350,12 @@
       <c r="J78" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K78">
+        <v>30</v>
+      </c>
+      <c r="L78" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -2926,6 +3388,12 @@
       <c r="J79" t="str">
         <v>Bank</v>
       </c>
+      <c r="K79">
+        <v>0</v>
+      </c>
+      <c r="L79" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -2958,6 +3426,12 @@
       <c r="J80" t="str">
         <v>Bank</v>
       </c>
+      <c r="K80">
+        <v>0</v>
+      </c>
+      <c r="L80" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -2990,6 +3464,12 @@
       <c r="J81" t="str">
         <v>Bank</v>
       </c>
+      <c r="K81">
+        <v>2</v>
+      </c>
+      <c r="L81" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -3016,6 +3496,12 @@
       <c r="H82" t="str">
         <v>Bank</v>
       </c>
+      <c r="K82">
+        <v>0</v>
+      </c>
+      <c r="L82" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -3048,6 +3534,12 @@
       <c r="J83" t="str">
         <v>Bank</v>
       </c>
+      <c r="K83">
+        <v>2</v>
+      </c>
+      <c r="L83" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -3080,6 +3572,12 @@
       <c r="J84" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K84">
+        <v>4</v>
+      </c>
+      <c r="L84" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -3112,6 +3610,12 @@
       <c r="J85" t="str">
         <v>Bank</v>
       </c>
+      <c r="K85">
+        <v>0</v>
+      </c>
+      <c r="L85" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -3144,6 +3648,12 @@
       <c r="J86" t="str">
         <v>Bank</v>
       </c>
+      <c r="K86">
+        <v>0</v>
+      </c>
+      <c r="L86" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -3176,6 +3686,12 @@
       <c r="J87" t="str">
         <v>Bank</v>
       </c>
+      <c r="K87">
+        <v>0</v>
+      </c>
+      <c r="L87" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -3208,6 +3724,12 @@
       <c r="J88" t="str">
         <v>Bank</v>
       </c>
+      <c r="K88">
+        <v>0</v>
+      </c>
+      <c r="L88" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -3240,6 +3762,12 @@
       <c r="J89" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K89">
+        <v>6</v>
+      </c>
+      <c r="L89" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -3272,6 +3800,12 @@
       <c r="J90" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K90">
+        <v>4</v>
+      </c>
+      <c r="L90" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -3304,6 +3838,12 @@
       <c r="J91" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K91">
+        <v>-2</v>
+      </c>
+      <c r="L91" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -3336,6 +3876,12 @@
       <c r="J92" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K92">
+        <v>2</v>
+      </c>
+      <c r="L92" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -3368,6 +3914,12 @@
       <c r="J93" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K93">
+        <v>22</v>
+      </c>
+      <c r="L93" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -3400,6 +3952,12 @@
       <c r="J94" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K94">
+        <v>2</v>
+      </c>
+      <c r="L94" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -3432,6 +3990,12 @@
       <c r="J95" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K95">
+        <v>8</v>
+      </c>
+      <c r="L95" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -3464,6 +4028,12 @@
       <c r="J96" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K96">
+        <v>10</v>
+      </c>
+      <c r="L96" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -3496,6 +4066,12 @@
       <c r="J97" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K97">
+        <v>2</v>
+      </c>
+      <c r="L97" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -3528,6 +4104,12 @@
       <c r="J98" t="str">
         <v>Bank</v>
       </c>
+      <c r="K98">
+        <v>0</v>
+      </c>
+      <c r="L98" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -3560,6 +4142,12 @@
       <c r="J99" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K99">
+        <v>13</v>
+      </c>
+      <c r="L99" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -3592,6 +4180,12 @@
       <c r="J100" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K100">
+        <v>6</v>
+      </c>
+      <c r="L100" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -3624,6 +4218,12 @@
       <c r="J101" t="str">
         <v>Bank</v>
       </c>
+      <c r="K101">
+        <v>0</v>
+      </c>
+      <c r="L101" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -3656,6 +4256,12 @@
       <c r="J102" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K102">
+        <v>20</v>
+      </c>
+      <c r="L102" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -3688,6 +4294,12 @@
       <c r="J103" t="str">
         <v>Bank</v>
       </c>
+      <c r="K103">
+        <v>0</v>
+      </c>
+      <c r="L103" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -3714,6 +4326,12 @@
       <c r="H104" t="str">
         <v>Bank</v>
       </c>
+      <c r="K104">
+        <v>0</v>
+      </c>
+      <c r="L104" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -3746,6 +4364,12 @@
       <c r="J105" t="str">
         <v>Bank</v>
       </c>
+      <c r="K105">
+        <v>0</v>
+      </c>
+      <c r="L105" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -3778,6 +4402,12 @@
       <c r="J106" t="str">
         <v>Bank</v>
       </c>
+      <c r="K106">
+        <v>2</v>
+      </c>
+      <c r="L106" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -3804,6 +4434,12 @@
       <c r="H107" t="str">
         <v>Bank</v>
       </c>
+      <c r="K107">
+        <v>0</v>
+      </c>
+      <c r="L107" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -3836,6 +4472,12 @@
       <c r="J108" t="str">
         <v>Bank</v>
       </c>
+      <c r="K108">
+        <v>0</v>
+      </c>
+      <c r="L108" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -3868,6 +4510,12 @@
       <c r="J109" t="str">
         <v>Bank</v>
       </c>
+      <c r="K109">
+        <v>0</v>
+      </c>
+      <c r="L109" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -3900,6 +4548,12 @@
       <c r="J110" t="str">
         <v>Bank</v>
       </c>
+      <c r="K110">
+        <v>0</v>
+      </c>
+      <c r="L110" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -3926,6 +4580,12 @@
       <c r="H111" t="str">
         <v>Bank</v>
       </c>
+      <c r="K111">
+        <v>0</v>
+      </c>
+      <c r="L111" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -3958,6 +4618,12 @@
       <c r="J112" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K112">
+        <v>6</v>
+      </c>
+      <c r="L112" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -3990,6 +4656,12 @@
       <c r="J113" t="str">
         <v>Bank</v>
       </c>
+      <c r="K113">
+        <v>0</v>
+      </c>
+      <c r="L113" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -4022,6 +4694,12 @@
       <c r="J114" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K114">
+        <v>11</v>
+      </c>
+      <c r="L114" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -4054,6 +4732,12 @@
       <c r="J115" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K115">
+        <v>0</v>
+      </c>
+      <c r="L115" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -4086,6 +4770,12 @@
       <c r="J116" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K116">
+        <v>20</v>
+      </c>
+      <c r="L116" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -4118,6 +4808,12 @@
       <c r="J117" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K117">
+        <v>6</v>
+      </c>
+      <c r="L117" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -4150,6 +4846,12 @@
       <c r="J118" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K118">
+        <v>4</v>
+      </c>
+      <c r="L118" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -4182,6 +4884,12 @@
       <c r="J119" t="str">
         <v>Bank</v>
       </c>
+      <c r="K119">
+        <v>6</v>
+      </c>
+      <c r="L119" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -4214,6 +4922,12 @@
       <c r="J120" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K120">
+        <v>6</v>
+      </c>
+      <c r="L120" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -4246,6 +4960,12 @@
       <c r="J121" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K121">
+        <v>2</v>
+      </c>
+      <c r="L121" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -4278,6 +4998,12 @@
       <c r="J122" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K122">
+        <v>16</v>
+      </c>
+      <c r="L122" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -4310,6 +5036,12 @@
       <c r="J123" t="str">
         <v>Bank</v>
       </c>
+      <c r="K123">
+        <v>0</v>
+      </c>
+      <c r="L123" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -4342,6 +5074,12 @@
       <c r="J124" t="str">
         <v>Bank</v>
       </c>
+      <c r="K124">
+        <v>0</v>
+      </c>
+      <c r="L124" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -4374,6 +5112,12 @@
       <c r="J125" t="str">
         <v>Bank</v>
       </c>
+      <c r="K125">
+        <v>0</v>
+      </c>
+      <c r="L125" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -4400,6 +5144,12 @@
       <c r="H126" t="str">
         <v>Bank</v>
       </c>
+      <c r="K126">
+        <v>0</v>
+      </c>
+      <c r="L126" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -4432,6 +5182,12 @@
       <c r="J127" t="str">
         <v>Bank</v>
       </c>
+      <c r="K127">
+        <v>0</v>
+      </c>
+      <c r="L127" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -4464,6 +5220,12 @@
       <c r="J128" t="str">
         <v>Bank</v>
       </c>
+      <c r="K128">
+        <v>2</v>
+      </c>
+      <c r="L128" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
@@ -4496,6 +5258,12 @@
       <c r="J129" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K129">
+        <v>12</v>
+      </c>
+      <c r="L129" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
@@ -4528,6 +5296,12 @@
       <c r="J130" t="str">
         <v>Bank</v>
       </c>
+      <c r="K130">
+        <v>0</v>
+      </c>
+      <c r="L130" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
@@ -4554,6 +5328,12 @@
       <c r="H131" t="str">
         <v>Bank</v>
       </c>
+      <c r="K131">
+        <v>0</v>
+      </c>
+      <c r="L131" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
@@ -4586,6 +5366,12 @@
       <c r="J132" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K132">
+        <v>0</v>
+      </c>
+      <c r="L132" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
@@ -4618,6 +5404,12 @@
       <c r="J133" t="str">
         <v>Bank</v>
       </c>
+      <c r="K133">
+        <v>2</v>
+      </c>
+      <c r="L133" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -4650,6 +5442,12 @@
       <c r="J134" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K134">
+        <v>0</v>
+      </c>
+      <c r="L134" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
@@ -4682,6 +5480,12 @@
       <c r="J135" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K135">
+        <v>-2</v>
+      </c>
+      <c r="L135" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
@@ -4714,6 +5518,12 @@
       <c r="J136" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K136">
+        <v>2</v>
+      </c>
+      <c r="L136" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
@@ -4746,6 +5556,12 @@
       <c r="J137" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K137">
+        <v>6</v>
+      </c>
+      <c r="L137" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
@@ -4778,6 +5594,12 @@
       <c r="J138" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K138">
+        <v>6</v>
+      </c>
+      <c r="L138" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
@@ -4810,6 +5632,12 @@
       <c r="J139" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K139">
+        <v>4</v>
+      </c>
+      <c r="L139" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
@@ -4842,6 +5670,12 @@
       <c r="J140" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K140">
+        <v>6</v>
+      </c>
+      <c r="L140" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
@@ -4874,6 +5708,12 @@
       <c r="J141" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K141">
+        <v>0</v>
+      </c>
+      <c r="L141" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
@@ -4906,6 +5746,12 @@
       <c r="J142" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K142">
+        <v>4</v>
+      </c>
+      <c r="L142" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
@@ -4938,6 +5784,12 @@
       <c r="J143" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K143">
+        <v>16</v>
+      </c>
+      <c r="L143" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
@@ -4970,6 +5822,12 @@
       <c r="J144" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K144">
+        <v>0</v>
+      </c>
+      <c r="L144" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
@@ -5002,6 +5860,12 @@
       <c r="J145" t="str">
         <v>Bank</v>
       </c>
+      <c r="K145">
+        <v>8</v>
+      </c>
+      <c r="L145" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
@@ -5034,6 +5898,12 @@
       <c r="J146" t="str">
         <v>Bank</v>
       </c>
+      <c r="K146">
+        <v>0</v>
+      </c>
+      <c r="L146" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
@@ -5066,6 +5936,12 @@
       <c r="J147" t="str">
         <v>Bank</v>
       </c>
+      <c r="K147">
+        <v>2</v>
+      </c>
+      <c r="L147" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
@@ -5098,6 +5974,12 @@
       <c r="J148" t="str">
         <v>Bank</v>
       </c>
+      <c r="K148">
+        <v>2</v>
+      </c>
+      <c r="L148" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
@@ -5130,6 +6012,12 @@
       <c r="J149" t="str">
         <v>Bank</v>
       </c>
+      <c r="K149">
+        <v>0</v>
+      </c>
+      <c r="L149" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
@@ -5162,6 +6050,12 @@
       <c r="J150" t="str">
         <v>Bank</v>
       </c>
+      <c r="K150">
+        <v>0</v>
+      </c>
+      <c r="L150" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
@@ -5194,6 +6088,12 @@
       <c r="J151" t="str">
         <v>Bank</v>
       </c>
+      <c r="K151">
+        <v>0</v>
+      </c>
+      <c r="L151" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
@@ -5226,6 +6126,12 @@
       <c r="J152" t="str">
         <v>Bank</v>
       </c>
+      <c r="K152">
+        <v>0</v>
+      </c>
+      <c r="L152" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
@@ -5258,6 +6164,12 @@
       <c r="J153" t="str">
         <v>Bank</v>
       </c>
+      <c r="K153">
+        <v>0</v>
+      </c>
+      <c r="L153" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
@@ -5290,6 +6202,12 @@
       <c r="J154" t="str">
         <v>Bank</v>
       </c>
+      <c r="K154">
+        <v>0</v>
+      </c>
+      <c r="L154" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
@@ -5322,6 +6240,12 @@
       <c r="J155" t="str">
         <v>Bank</v>
       </c>
+      <c r="K155">
+        <v>0</v>
+      </c>
+      <c r="L155" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
@@ -5354,6 +6278,12 @@
       <c r="J156" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K156">
+        <v>10</v>
+      </c>
+      <c r="L156" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
@@ -5386,6 +6316,12 @@
       <c r="J157" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K157">
+        <v>2</v>
+      </c>
+      <c r="L157" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
@@ -5418,6 +6354,12 @@
       <c r="J158" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K158">
+        <v>0</v>
+      </c>
+      <c r="L158" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
@@ -5450,6 +6392,12 @@
       <c r="J159" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K159">
+        <v>2</v>
+      </c>
+      <c r="L159" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
@@ -5482,6 +6430,12 @@
       <c r="J160" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K160">
+        <v>-2</v>
+      </c>
+      <c r="L160" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
@@ -5514,6 +6468,12 @@
       <c r="J161" t="str">
         <v>Bank</v>
       </c>
+      <c r="K161">
+        <v>10</v>
+      </c>
+      <c r="L161" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
@@ -5546,6 +6506,12 @@
       <c r="J162" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K162">
+        <v>4</v>
+      </c>
+      <c r="L162" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
@@ -5578,6 +6544,12 @@
       <c r="J163" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K163">
+        <v>4</v>
+      </c>
+      <c r="L163" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
@@ -5610,6 +6582,12 @@
       <c r="J164" t="str">
         <v>Bank</v>
       </c>
+      <c r="K164">
+        <v>9</v>
+      </c>
+      <c r="L164" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
@@ -5642,6 +6620,12 @@
       <c r="J165" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K165">
+        <v>13</v>
+      </c>
+      <c r="L165" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
@@ -5674,6 +6658,12 @@
       <c r="J166" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K166">
+        <v>7</v>
+      </c>
+      <c r="L166" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
@@ -5706,6 +6696,12 @@
       <c r="J167" t="str">
         <v>Bank</v>
       </c>
+      <c r="K167">
+        <v>0</v>
+      </c>
+      <c r="L167" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
@@ -5738,6 +6734,12 @@
       <c r="J168" t="str">
         <v>Bank</v>
       </c>
+      <c r="K168">
+        <v>0</v>
+      </c>
+      <c r="L168" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
@@ -5770,6 +6772,12 @@
       <c r="J169" t="str">
         <v>Bank</v>
       </c>
+      <c r="K169">
+        <v>0</v>
+      </c>
+      <c r="L169" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
@@ -5802,6 +6810,12 @@
       <c r="J170" t="str">
         <v>Bank</v>
       </c>
+      <c r="K170">
+        <v>2</v>
+      </c>
+      <c r="L170" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
@@ -5834,6 +6848,12 @@
       <c r="J171" t="str">
         <v>Bank</v>
       </c>
+      <c r="K171">
+        <v>0</v>
+      </c>
+      <c r="L171" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
@@ -5866,6 +6886,12 @@
       <c r="J172" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K172">
+        <v>0</v>
+      </c>
+      <c r="L172" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
@@ -5898,6 +6924,12 @@
       <c r="J173" t="str">
         <v>Bank</v>
       </c>
+      <c r="K173">
+        <v>0</v>
+      </c>
+      <c r="L173" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
@@ -5930,6 +6962,12 @@
       <c r="J174" t="str">
         <v>Bank</v>
       </c>
+      <c r="K174">
+        <v>0</v>
+      </c>
+      <c r="L174" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
@@ -5962,6 +7000,12 @@
       <c r="J175" t="str">
         <v>Bank</v>
       </c>
+      <c r="K175">
+        <v>0</v>
+      </c>
+      <c r="L175" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
@@ -5994,6 +7038,12 @@
       <c r="J176" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K176">
+        <v>2</v>
+      </c>
+      <c r="L176" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
@@ -6026,6 +7076,12 @@
       <c r="J177" t="str">
         <v>Bank</v>
       </c>
+      <c r="K177">
+        <v>0</v>
+      </c>
+      <c r="L177" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
@@ -6058,6 +7114,12 @@
       <c r="J178" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K178">
+        <v>8</v>
+      </c>
+      <c r="L178" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
@@ -6090,6 +7152,12 @@
       <c r="J179" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K179">
+        <v>0</v>
+      </c>
+      <c r="L179" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
@@ -6122,6 +7190,12 @@
       <c r="J180" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K180">
+        <v>6</v>
+      </c>
+      <c r="L180" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
@@ -6154,6 +7228,12 @@
       <c r="J181" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K181">
+        <v>2</v>
+      </c>
+      <c r="L181" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
@@ -6186,6 +7266,12 @@
       <c r="J182" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K182">
+        <v>2</v>
+      </c>
+      <c r="L182" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
@@ -6218,6 +7304,12 @@
       <c r="J183" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K183">
+        <v>6</v>
+      </c>
+      <c r="L183" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
@@ -6250,6 +7342,12 @@
       <c r="J184" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K184">
+        <v>2</v>
+      </c>
+      <c r="L184" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
@@ -6282,6 +7380,12 @@
       <c r="J185" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K185">
+        <v>4</v>
+      </c>
+      <c r="L185" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
@@ -6314,6 +7418,12 @@
       <c r="J186" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K186">
+        <v>0</v>
+      </c>
+      <c r="L186" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
@@ -6346,6 +7456,12 @@
       <c r="J187" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K187">
+        <v>0</v>
+      </c>
+      <c r="L187" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
@@ -6378,6 +7494,12 @@
       <c r="J188" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K188">
+        <v>-2</v>
+      </c>
+      <c r="L188" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
@@ -6410,6 +7532,12 @@
       <c r="J189" t="str">
         <v>Bank</v>
       </c>
+      <c r="K189">
+        <v>0</v>
+      </c>
+      <c r="L189" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
@@ -6442,6 +7570,12 @@
       <c r="J190" t="str">
         <v>Bank</v>
       </c>
+      <c r="K190">
+        <v>0</v>
+      </c>
+      <c r="L190" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
@@ -6474,6 +7608,12 @@
       <c r="J191" t="str">
         <v>Bank</v>
       </c>
+      <c r="K191">
+        <v>0</v>
+      </c>
+      <c r="L191" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
@@ -6506,6 +7646,12 @@
       <c r="J192" t="str">
         <v>Bank</v>
       </c>
+      <c r="K192">
+        <v>0</v>
+      </c>
+      <c r="L192" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
@@ -6532,6 +7678,12 @@
       <c r="H193" t="str">
         <v>Bank</v>
       </c>
+      <c r="K193">
+        <v>0</v>
+      </c>
+      <c r="L193" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
@@ -6564,6 +7716,12 @@
       <c r="J194" t="str">
         <v>Bank</v>
       </c>
+      <c r="K194">
+        <v>0</v>
+      </c>
+      <c r="L194" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
@@ -6596,6 +7754,12 @@
       <c r="J195" t="str">
         <v>Bank</v>
       </c>
+      <c r="K195">
+        <v>0</v>
+      </c>
+      <c r="L195" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
@@ -6628,6 +7792,12 @@
       <c r="J196" t="str">
         <v>Bank</v>
       </c>
+      <c r="K196">
+        <v>0</v>
+      </c>
+      <c r="L196" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
@@ -6660,6 +7830,12 @@
       <c r="J197" t="str">
         <v>Bank</v>
       </c>
+      <c r="K197">
+        <v>2</v>
+      </c>
+      <c r="L197" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
@@ -6686,6 +7862,12 @@
       <c r="H198" t="str">
         <v>Bank</v>
       </c>
+      <c r="K198">
+        <v>0</v>
+      </c>
+      <c r="L198" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
@@ -6718,6 +7900,12 @@
       <c r="J199" t="str">
         <v>Bank</v>
       </c>
+      <c r="K199">
+        <v>0</v>
+      </c>
+      <c r="L199" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
@@ -6750,6 +7938,12 @@
       <c r="J200" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K200">
+        <v>6</v>
+      </c>
+      <c r="L200" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
@@ -6782,6 +7976,12 @@
       <c r="J201" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K201">
+        <v>6</v>
+      </c>
+      <c r="L201" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
@@ -6814,6 +8014,12 @@
       <c r="J202" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K202">
+        <v>22</v>
+      </c>
+      <c r="L202" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
@@ -6846,6 +8052,12 @@
       <c r="J203" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K203">
+        <v>0</v>
+      </c>
+      <c r="L203" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
@@ -6878,6 +8090,12 @@
       <c r="J204" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K204">
+        <v>6</v>
+      </c>
+      <c r="L204" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
@@ -6910,6 +8128,12 @@
       <c r="J205" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K205">
+        <v>4</v>
+      </c>
+      <c r="L205" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
@@ -6942,6 +8166,12 @@
       <c r="J206" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K206">
+        <v>4</v>
+      </c>
+      <c r="L206" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
@@ -6974,6 +8204,12 @@
       <c r="J207" t="str">
         <v>Bank</v>
       </c>
+      <c r="K207">
+        <v>0</v>
+      </c>
+      <c r="L207" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
@@ -7006,6 +8242,12 @@
       <c r="J208" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K208">
+        <v>4</v>
+      </c>
+      <c r="L208" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
@@ -7038,6 +8280,12 @@
       <c r="J209" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K209">
+        <v>6</v>
+      </c>
+      <c r="L209" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
@@ -7070,6 +8318,12 @@
       <c r="J210" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K210">
+        <v>13</v>
+      </c>
+      <c r="L210" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
@@ -7102,6 +8356,12 @@
       <c r="J211" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K211">
+        <v>12</v>
+      </c>
+      <c r="L211" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
@@ -7134,6 +8394,12 @@
       <c r="J212" t="str">
         <v>Bank</v>
       </c>
+      <c r="K212">
+        <v>2</v>
+      </c>
+      <c r="L212" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
@@ -7166,6 +8432,12 @@
       <c r="J213" t="str">
         <v>Bank</v>
       </c>
+      <c r="K213">
+        <v>2</v>
+      </c>
+      <c r="L213" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
@@ -7198,6 +8470,12 @@
       <c r="J214" t="str">
         <v>Bank</v>
       </c>
+      <c r="K214">
+        <v>0</v>
+      </c>
+      <c r="L214" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
@@ -7230,6 +8508,12 @@
       <c r="J215" t="str">
         <v>Bank</v>
       </c>
+      <c r="K215">
+        <v>0</v>
+      </c>
+      <c r="L215" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
@@ -7262,6 +8546,12 @@
       <c r="J216" t="str">
         <v>Bank</v>
       </c>
+      <c r="K216">
+        <v>2</v>
+      </c>
+      <c r="L216" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
@@ -7294,6 +8584,12 @@
       <c r="J217" t="str">
         <v>Bank</v>
       </c>
+      <c r="K217">
+        <v>0</v>
+      </c>
+      <c r="L217" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
@@ -7326,6 +8622,12 @@
       <c r="J218" t="str">
         <v>Bank</v>
       </c>
+      <c r="K218">
+        <v>0</v>
+      </c>
+      <c r="L218" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
@@ -7358,6 +8660,12 @@
       <c r="J219" t="str">
         <v>Bank</v>
       </c>
+      <c r="K219">
+        <v>0</v>
+      </c>
+      <c r="L219" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
@@ -7390,6 +8698,12 @@
       <c r="J220" t="str">
         <v>Bank</v>
       </c>
+      <c r="K220">
+        <v>0</v>
+      </c>
+      <c r="L220" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
@@ -7422,6 +8736,12 @@
       <c r="J221" t="str">
         <v>Bank</v>
       </c>
+      <c r="K221">
+        <v>0</v>
+      </c>
+      <c r="L221" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
@@ -7454,6 +8774,12 @@
       <c r="J222" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K222">
+        <v>8</v>
+      </c>
+      <c r="L222" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
@@ -7486,6 +8812,12 @@
       <c r="J223" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K223">
+        <v>6</v>
+      </c>
+      <c r="L223" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
@@ -7518,6 +8850,12 @@
       <c r="J224" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K224">
+        <v>0</v>
+      </c>
+      <c r="L224" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
@@ -7550,6 +8888,12 @@
       <c r="J225" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K225">
+        <v>2</v>
+      </c>
+      <c r="L225" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
@@ -7582,6 +8926,12 @@
       <c r="J226" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K226">
+        <v>4</v>
+      </c>
+      <c r="L226" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
@@ -7614,6 +8964,12 @@
       <c r="J227" t="str">
         <v>Bank</v>
       </c>
+      <c r="K227">
+        <v>0</v>
+      </c>
+      <c r="L227" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
@@ -7646,6 +9002,12 @@
       <c r="J228" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K228">
+        <v>4</v>
+      </c>
+      <c r="L228" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
@@ -7678,6 +9040,12 @@
       <c r="J229" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K229">
+        <v>6</v>
+      </c>
+      <c r="L229" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
@@ -7710,6 +9078,12 @@
       <c r="J230" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K230">
+        <v>13</v>
+      </c>
+      <c r="L230" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
@@ -7742,6 +9116,12 @@
       <c r="J231" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K231">
+        <v>7</v>
+      </c>
+      <c r="L231" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
@@ -7774,6 +9154,12 @@
       <c r="J232" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K232">
+        <v>0</v>
+      </c>
+      <c r="L232" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
@@ -7806,6 +9192,12 @@
       <c r="J233" t="str">
         <v>Startelf</v>
       </c>
+      <c r="K233">
+        <v>2</v>
+      </c>
+      <c r="L233" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
@@ -7838,6 +9230,12 @@
       <c r="J234" t="str">
         <v>Bank</v>
       </c>
+      <c r="K234">
+        <v>2</v>
+      </c>
+      <c r="L234" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
@@ -7870,6 +9268,12 @@
       <c r="J235" t="str">
         <v>Bank</v>
       </c>
+      <c r="K235">
+        <v>0</v>
+      </c>
+      <c r="L235" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
@@ -7902,6 +9306,12 @@
       <c r="J236" t="str">
         <v>Bank</v>
       </c>
+      <c r="K236">
+        <v>0</v>
+      </c>
+      <c r="L236" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
@@ -7934,6 +9344,12 @@
       <c r="J237" t="str">
         <v>Bank</v>
       </c>
+      <c r="K237">
+        <v>0</v>
+      </c>
+      <c r="L237" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
@@ -7966,6 +9382,12 @@
       <c r="J238" t="str">
         <v>Bank</v>
       </c>
+      <c r="K238">
+        <v>0</v>
+      </c>
+      <c r="L238" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
@@ -7998,6 +9420,12 @@
       <c r="J239" t="str">
         <v>Bank</v>
       </c>
+      <c r="K239">
+        <v>0</v>
+      </c>
+      <c r="L239" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
@@ -8030,6 +9458,12 @@
       <c r="J240" t="str">
         <v>Bank</v>
       </c>
+      <c r="K240">
+        <v>0</v>
+      </c>
+      <c r="L240" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
@@ -8062,6 +9496,12 @@
       <c r="J241" t="str">
         <v>Bank</v>
       </c>
+      <c r="K241">
+        <v>0</v>
+      </c>
+      <c r="L241" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
@@ -8094,6 +9534,12 @@
       <c r="J242" t="str">
         <v>Bank</v>
       </c>
+      <c r="K242">
+        <v>6</v>
+      </c>
+      <c r="L242" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
@@ -8124,6 +9570,12 @@
         <v>-6</v>
       </c>
       <c r="J243" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="K243">
+        <v>0</v>
+      </c>
+      <c r="L243" t="str">
         <v>Bank</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Spieltag 4: Datendateien der Vergleichszentrale nachgezogen (Kicker-Korrektur Tietz)
saison.xlsx, spieltagspunkte.csv, historie/manager.json und stats/powerverlauf.json
lagen noch auf dem Stand vor der Kicker-Korrektur (Tietz -2 Punkte bei 5 Managern).
Der vorige Commit hatte nur die Manager-/Portal-Seiten aktualisiert, nicht die
Rohdaten, aus denen die Vergleichszentrale (generator/vergleich.html) selbst laedt.
</commit_message>
<xml_diff>
--- a/saison.xlsx
+++ b/saison.xlsx
@@ -855,7 +855,7 @@
         <v>Startelf</v>
       </c>
       <c r="K12">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L12" t="str">
         <v>Startelf</v>
@@ -2477,7 +2477,7 @@
         <v>Startelf</v>
       </c>
       <c r="K55">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L55" t="str">
         <v>Startelf</v>
@@ -3275,7 +3275,7 @@
         <v>Startelf</v>
       </c>
       <c r="K76">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L76" t="str">
         <v>Startelf</v>
@@ -6659,7 +6659,7 @@
         <v>Startelf</v>
       </c>
       <c r="K166">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L166" t="str">
         <v>Startelf</v>
@@ -9117,7 +9117,7 @@
         <v>Startelf</v>
       </c>
       <c r="K231">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L231" t="str">
         <v>Startelf</v>

</xml_diff>

<commit_message>
Spieltag 5 (2026/27): Daten, Kaderseiten und Portal-Tabelle aktualisiert
- Datendateien aus D:\Spreeliga\stand aufgefrischt: saison.xlsx, players-se.csv,
  spieltagspunkte.csv, clientdb.json, historie/manager.json, stats/saison.json,
  neu stats/st5.json, stats/powerverlauf.json.
- Alle 11 manager-*.html und portal.html mit werkstatt\bauen\website.js erzeugt.
- Erzeugt von werkstatt\spieltag.js; der Lauf vom 12.10.2026 brach beim git add ab
  (OneDrive sperrte eine Datei in .git/objects), die Dateien lagen aber schon richtig
  im Repo. Hier nur nachgeholt.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/saison.xlsx
+++ b/saison.xlsx
@@ -480,6 +480,12 @@
       <c r="L2" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M2">
+        <v>6</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -518,6 +524,12 @@
       <c r="L3" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -556,6 +568,12 @@
       <c r="L4" t="str">
         <v>Bank</v>
       </c>
+      <c r="M4">
+        <v>4</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -594,6 +612,12 @@
       <c r="L5" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M5">
+        <v>6</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -632,6 +656,12 @@
       <c r="L6" t="str">
         <v>Bank</v>
       </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -670,6 +700,12 @@
       <c r="L7" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -708,6 +744,12 @@
       <c r="L8" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M8">
+        <v>8</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -746,6 +788,12 @@
       <c r="L9" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -784,6 +832,12 @@
       <c r="L10" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M10">
+        <v>2</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -822,6 +876,12 @@
       <c r="L11" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M11">
+        <v>-2</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -860,6 +920,12 @@
       <c r="L12" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -898,6 +964,12 @@
       <c r="L13" t="str">
         <v>Bank</v>
       </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -936,6 +1008,12 @@
       <c r="L14" t="str">
         <v>Bank</v>
       </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -974,6 +1052,12 @@
       <c r="L15" t="str">
         <v>Bank</v>
       </c>
+      <c r="M15">
+        <v>2</v>
+      </c>
+      <c r="N15" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1012,6 +1096,12 @@
       <c r="L16" t="str">
         <v>Bank</v>
       </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="N16" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1050,6 +1140,12 @@
       <c r="L17" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M17">
+        <v>3</v>
+      </c>
+      <c r="N17" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1088,6 +1184,12 @@
       <c r="L18" t="str">
         <v>Bank</v>
       </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1126,6 +1228,12 @@
       <c r="L19" t="str">
         <v>Bank</v>
       </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1164,6 +1272,12 @@
       <c r="L20" t="str">
         <v>Bank</v>
       </c>
+      <c r="M20">
+        <v>2</v>
+      </c>
+      <c r="N20" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1202,6 +1316,12 @@
       <c r="L21" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M21">
+        <v>6</v>
+      </c>
+      <c r="N21" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1240,6 +1360,12 @@
       <c r="L22" t="str">
         <v>Bank</v>
       </c>
+      <c r="M22">
+        <v>0</v>
+      </c>
+      <c r="N22" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1278,6 +1404,12 @@
       <c r="L23" t="str">
         <v>Bank</v>
       </c>
+      <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="N23" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1316,6 +1448,12 @@
       <c r="L24" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M24">
+        <v>8</v>
+      </c>
+      <c r="N24" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1354,6 +1492,12 @@
       <c r="L25" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M25">
+        <v>2</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1386,6 +1530,12 @@
       <c r="L26" t="str">
         <v>Bank</v>
       </c>
+      <c r="M26">
+        <v>0</v>
+      </c>
+      <c r="N26" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1424,6 +1574,12 @@
       <c r="L27" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M27">
+        <v>0</v>
+      </c>
+      <c r="N27" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1462,6 +1618,12 @@
       <c r="L28" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M28">
+        <v>10</v>
+      </c>
+      <c r="N28" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1500,6 +1662,12 @@
       <c r="L29" t="str">
         <v>Bank</v>
       </c>
+      <c r="M29">
+        <v>0</v>
+      </c>
+      <c r="N29" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1538,6 +1706,12 @@
       <c r="L30" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M30">
+        <v>8</v>
+      </c>
+      <c r="N30" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1576,6 +1750,12 @@
       <c r="L31" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M31">
+        <v>2</v>
+      </c>
+      <c r="N31" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1614,6 +1794,12 @@
       <c r="L32" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M32">
+        <v>2</v>
+      </c>
+      <c r="N32" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1652,6 +1838,12 @@
       <c r="L33" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M33">
+        <v>17</v>
+      </c>
+      <c r="N33" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1690,6 +1882,12 @@
       <c r="L34" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M34">
+        <v>11</v>
+      </c>
+      <c r="N34" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1728,6 +1926,12 @@
       <c r="L35" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M35">
+        <v>0</v>
+      </c>
+      <c r="N35" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1766,6 +1970,12 @@
       <c r="L36" t="str">
         <v>Bank</v>
       </c>
+      <c r="M36">
+        <v>0</v>
+      </c>
+      <c r="N36" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1804,6 +2014,12 @@
       <c r="L37" t="str">
         <v>Bank</v>
       </c>
+      <c r="M37">
+        <v>0</v>
+      </c>
+      <c r="N37" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -1842,6 +2058,12 @@
       <c r="L38" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M38">
+        <v>0</v>
+      </c>
+      <c r="N38" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1880,6 +2102,12 @@
       <c r="L39" t="str">
         <v>Bank</v>
       </c>
+      <c r="M39">
+        <v>2</v>
+      </c>
+      <c r="N39" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1918,6 +2146,12 @@
       <c r="L40" t="str">
         <v>Bank</v>
       </c>
+      <c r="M40">
+        <v>0</v>
+      </c>
+      <c r="N40" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1956,6 +2190,12 @@
       <c r="L41" t="str">
         <v>Bank</v>
       </c>
+      <c r="M41">
+        <v>0</v>
+      </c>
+      <c r="N41" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -1994,6 +2234,12 @@
       <c r="L42" t="str">
         <v>Bank</v>
       </c>
+      <c r="M42">
+        <v>0</v>
+      </c>
+      <c r="N42" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -2026,6 +2272,12 @@
       <c r="L43" t="str">
         <v>Bank</v>
       </c>
+      <c r="M43">
+        <v>0</v>
+      </c>
+      <c r="N43" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -2064,6 +2316,12 @@
       <c r="L44" t="str">
         <v>Bank</v>
       </c>
+      <c r="M44">
+        <v>0</v>
+      </c>
+      <c r="N44" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -2102,6 +2360,12 @@
       <c r="L45" t="str">
         <v>Bank</v>
       </c>
+      <c r="M45">
+        <v>2</v>
+      </c>
+      <c r="N45" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -2140,6 +2404,12 @@
       <c r="L46" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M46">
+        <v>6</v>
+      </c>
+      <c r="N46" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -2178,6 +2448,12 @@
       <c r="L47" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M47">
+        <v>7</v>
+      </c>
+      <c r="N47" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -2216,6 +2492,12 @@
       <c r="L48" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M48">
+        <v>-2</v>
+      </c>
+      <c r="N48" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -2254,6 +2536,12 @@
       <c r="L49" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M49">
+        <v>4</v>
+      </c>
+      <c r="N49" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -2292,6 +2580,12 @@
       <c r="L50" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M50">
+        <v>8</v>
+      </c>
+      <c r="N50" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -2330,6 +2624,12 @@
       <c r="L51" t="str">
         <v>Bank</v>
       </c>
+      <c r="M51">
+        <v>0</v>
+      </c>
+      <c r="N51" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -2368,6 +2668,12 @@
       <c r="L52" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M52">
+        <v>2</v>
+      </c>
+      <c r="N52" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -2406,6 +2712,12 @@
       <c r="L53" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M53">
+        <v>2</v>
+      </c>
+      <c r="N53" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -2444,6 +2756,12 @@
       <c r="L54" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M54">
+        <v>2</v>
+      </c>
+      <c r="N54" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -2482,6 +2800,12 @@
       <c r="L55" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M55">
+        <v>0</v>
+      </c>
+      <c r="N55" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2520,6 +2844,12 @@
       <c r="L56" t="str">
         <v>Bank</v>
       </c>
+      <c r="M56">
+        <v>0</v>
+      </c>
+      <c r="N56" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2558,6 +2888,12 @@
       <c r="L57" t="str">
         <v>Bank</v>
       </c>
+      <c r="M57">
+        <v>0</v>
+      </c>
+      <c r="N57" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -2596,6 +2932,12 @@
       <c r="L58" t="str">
         <v>Bank</v>
       </c>
+      <c r="M58">
+        <v>0</v>
+      </c>
+      <c r="N58" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2634,6 +2976,12 @@
       <c r="L59" t="str">
         <v>Bank</v>
       </c>
+      <c r="M59">
+        <v>0</v>
+      </c>
+      <c r="N59" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -2672,6 +3020,12 @@
       <c r="L60" t="str">
         <v>Bank</v>
       </c>
+      <c r="M60">
+        <v>2</v>
+      </c>
+      <c r="N60" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -2710,6 +3064,12 @@
       <c r="L61" t="str">
         <v>Bank</v>
       </c>
+      <c r="M61">
+        <v>2</v>
+      </c>
+      <c r="N61" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -2748,6 +3108,12 @@
       <c r="L62" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M62">
+        <v>0</v>
+      </c>
+      <c r="N62" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -2786,6 +3152,12 @@
       <c r="L63" t="str">
         <v>Bank</v>
       </c>
+      <c r="M63">
+        <v>0</v>
+      </c>
+      <c r="N63" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -2824,6 +3196,12 @@
       <c r="L64" t="str">
         <v>Bank</v>
       </c>
+      <c r="M64">
+        <v>0</v>
+      </c>
+      <c r="N64" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -2862,6 +3240,12 @@
       <c r="L65" t="str">
         <v>Bank</v>
       </c>
+      <c r="M65">
+        <v>2</v>
+      </c>
+      <c r="N65" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -2900,6 +3284,12 @@
       <c r="L66" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M66">
+        <v>2</v>
+      </c>
+      <c r="N66" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -2938,6 +3328,12 @@
       <c r="L67" t="str">
         <v>Bank</v>
       </c>
+      <c r="M67">
+        <v>0</v>
+      </c>
+      <c r="N67" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -2976,6 +3372,12 @@
       <c r="L68" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M68">
+        <v>8</v>
+      </c>
+      <c r="N68" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -3014,6 +3416,12 @@
       <c r="L69" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M69">
+        <v>6</v>
+      </c>
+      <c r="N69" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -3052,6 +3460,12 @@
       <c r="L70" t="str">
         <v>Bank</v>
       </c>
+      <c r="M70">
+        <v>4</v>
+      </c>
+      <c r="N70" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -3090,6 +3504,12 @@
       <c r="L71" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M71">
+        <v>2</v>
+      </c>
+      <c r="N71" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -3128,6 +3548,12 @@
       <c r="L72" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M72">
+        <v>0</v>
+      </c>
+      <c r="N72" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -3166,6 +3592,12 @@
       <c r="L73" t="str">
         <v>Bank</v>
       </c>
+      <c r="M73">
+        <v>0</v>
+      </c>
+      <c r="N73" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -3204,6 +3636,12 @@
       <c r="L74" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M74">
+        <v>4</v>
+      </c>
+      <c r="N74" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -3242,6 +3680,12 @@
       <c r="L75" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M75">
+        <v>2</v>
+      </c>
+      <c r="N75" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -3280,6 +3724,12 @@
       <c r="L76" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M76">
+        <v>0</v>
+      </c>
+      <c r="N76" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -3318,6 +3768,12 @@
       <c r="L77" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M77">
+        <v>4</v>
+      </c>
+      <c r="N77" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -3356,6 +3812,12 @@
       <c r="L78" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M78">
+        <v>2</v>
+      </c>
+      <c r="N78" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -3394,6 +3856,12 @@
       <c r="L79" t="str">
         <v>Bank</v>
       </c>
+      <c r="M79">
+        <v>0</v>
+      </c>
+      <c r="N79" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -3432,6 +3900,12 @@
       <c r="L80" t="str">
         <v>Bank</v>
       </c>
+      <c r="M80">
+        <v>0</v>
+      </c>
+      <c r="N80" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -3470,6 +3944,12 @@
       <c r="L81" t="str">
         <v>Bank</v>
       </c>
+      <c r="M81">
+        <v>2</v>
+      </c>
+      <c r="N81" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -3502,6 +3982,12 @@
       <c r="L82" t="str">
         <v>Bank</v>
       </c>
+      <c r="M82">
+        <v>0</v>
+      </c>
+      <c r="N82" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -3540,6 +4026,12 @@
       <c r="L83" t="str">
         <v>Bank</v>
       </c>
+      <c r="M83">
+        <v>2</v>
+      </c>
+      <c r="N83" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -3578,6 +4070,12 @@
       <c r="L84" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M84">
+        <v>6</v>
+      </c>
+      <c r="N84" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -3616,6 +4114,12 @@
       <c r="L85" t="str">
         <v>Bank</v>
       </c>
+      <c r="M85">
+        <v>0</v>
+      </c>
+      <c r="N85" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -3654,6 +4158,12 @@
       <c r="L86" t="str">
         <v>Bank</v>
       </c>
+      <c r="M86">
+        <v>0</v>
+      </c>
+      <c r="N86" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -3692,6 +4202,12 @@
       <c r="L87" t="str">
         <v>Bank</v>
       </c>
+      <c r="M87">
+        <v>0</v>
+      </c>
+      <c r="N87" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -3730,6 +4246,12 @@
       <c r="L88" t="str">
         <v>Bank</v>
       </c>
+      <c r="M88">
+        <v>0</v>
+      </c>
+      <c r="N88" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -3768,6 +4290,12 @@
       <c r="L89" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M89">
+        <v>4</v>
+      </c>
+      <c r="N89" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -3806,6 +4334,12 @@
       <c r="L90" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M90">
+        <v>4</v>
+      </c>
+      <c r="N90" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -3844,6 +4378,12 @@
       <c r="L91" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M91">
+        <v>-2</v>
+      </c>
+      <c r="N91" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -3882,6 +4422,12 @@
       <c r="L92" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M92">
+        <v>7</v>
+      </c>
+      <c r="N92" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -3920,6 +4466,12 @@
       <c r="L93" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M93">
+        <v>2</v>
+      </c>
+      <c r="N93" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -3958,6 +4510,12 @@
       <c r="L94" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M94">
+        <v>0</v>
+      </c>
+      <c r="N94" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -3996,6 +4554,12 @@
       <c r="L95" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M95">
+        <v>8</v>
+      </c>
+      <c r="N95" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -4034,6 +4598,12 @@
       <c r="L96" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M96">
+        <v>6</v>
+      </c>
+      <c r="N96" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -4072,6 +4642,12 @@
       <c r="L97" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M97">
+        <v>2</v>
+      </c>
+      <c r="N97" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -4110,6 +4686,12 @@
       <c r="L98" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M98">
+        <v>4</v>
+      </c>
+      <c r="N98" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -4148,6 +4730,12 @@
       <c r="L99" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M99">
+        <v>-2</v>
+      </c>
+      <c r="N99" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -4186,6 +4774,12 @@
       <c r="L100" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M100">
+        <v>4</v>
+      </c>
+      <c r="N100" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -4224,6 +4818,12 @@
       <c r="L101" t="str">
         <v>Bank</v>
       </c>
+      <c r="M101">
+        <v>0</v>
+      </c>
+      <c r="N101" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -4262,6 +4862,12 @@
       <c r="L102" t="str">
         <v>Bank</v>
       </c>
+      <c r="M102">
+        <v>6</v>
+      </c>
+      <c r="N102" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -4300,6 +4906,12 @@
       <c r="L103" t="str">
         <v>Bank</v>
       </c>
+      <c r="M103">
+        <v>2</v>
+      </c>
+      <c r="N103" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -4332,6 +4944,12 @@
       <c r="L104" t="str">
         <v>Bank</v>
       </c>
+      <c r="M104">
+        <v>0</v>
+      </c>
+      <c r="N104" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -4370,6 +4988,12 @@
       <c r="L105" t="str">
         <v>Bank</v>
       </c>
+      <c r="M105">
+        <v>0</v>
+      </c>
+      <c r="N105" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -4408,6 +5032,12 @@
       <c r="L106" t="str">
         <v>Bank</v>
       </c>
+      <c r="M106">
+        <v>2</v>
+      </c>
+      <c r="N106" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -4440,6 +5070,12 @@
       <c r="L107" t="str">
         <v>Bank</v>
       </c>
+      <c r="M107">
+        <v>0</v>
+      </c>
+      <c r="N107" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -4478,6 +5114,12 @@
       <c r="L108" t="str">
         <v>Bank</v>
       </c>
+      <c r="M108">
+        <v>0</v>
+      </c>
+      <c r="N108" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -4516,6 +5158,12 @@
       <c r="L109" t="str">
         <v>Bank</v>
       </c>
+      <c r="M109">
+        <v>0</v>
+      </c>
+      <c r="N109" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -4554,6 +5202,12 @@
       <c r="L110" t="str">
         <v>Bank</v>
       </c>
+      <c r="M110">
+        <v>0</v>
+      </c>
+      <c r="N110" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -4586,6 +5240,12 @@
       <c r="L111" t="str">
         <v>Bank</v>
       </c>
+      <c r="M111">
+        <v>0</v>
+      </c>
+      <c r="N111" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -4624,6 +5284,12 @@
       <c r="L112" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M112">
+        <v>4</v>
+      </c>
+      <c r="N112" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -4662,6 +5328,12 @@
       <c r="L113" t="str">
         <v>Bank</v>
       </c>
+      <c r="M113">
+        <v>2</v>
+      </c>
+      <c r="N113" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -4700,6 +5372,12 @@
       <c r="L114" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M114">
+        <v>2</v>
+      </c>
+      <c r="N114" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -4738,6 +5416,12 @@
       <c r="L115" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M115">
+        <v>6</v>
+      </c>
+      <c r="N115" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -4776,6 +5460,12 @@
       <c r="L116" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M116">
+        <v>8</v>
+      </c>
+      <c r="N116" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -4814,6 +5504,12 @@
       <c r="L117" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M117">
+        <v>6</v>
+      </c>
+      <c r="N117" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -4852,6 +5548,12 @@
       <c r="L118" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M118">
+        <v>8</v>
+      </c>
+      <c r="N118" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -4890,6 +5592,12 @@
       <c r="L119" t="str">
         <v>Bank</v>
       </c>
+      <c r="M119">
+        <v>6</v>
+      </c>
+      <c r="N119" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -4928,6 +5636,12 @@
       <c r="L120" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M120">
+        <v>10</v>
+      </c>
+      <c r="N120" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -4966,6 +5680,12 @@
       <c r="L121" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M121">
+        <v>0</v>
+      </c>
+      <c r="N121" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -5004,6 +5724,12 @@
       <c r="L122" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M122">
+        <v>17</v>
+      </c>
+      <c r="N122" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -5042,6 +5768,12 @@
       <c r="L123" t="str">
         <v>Bank</v>
       </c>
+      <c r="M123">
+        <v>0</v>
+      </c>
+      <c r="N123" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -5080,6 +5812,12 @@
       <c r="L124" t="str">
         <v>Bank</v>
       </c>
+      <c r="M124">
+        <v>0</v>
+      </c>
+      <c r="N124" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -5118,6 +5856,12 @@
       <c r="L125" t="str">
         <v>Bank</v>
       </c>
+      <c r="M125">
+        <v>0</v>
+      </c>
+      <c r="N125" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -5150,6 +5894,12 @@
       <c r="L126" t="str">
         <v>Bank</v>
       </c>
+      <c r="M126">
+        <v>0</v>
+      </c>
+      <c r="N126" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -5188,6 +5938,12 @@
       <c r="L127" t="str">
         <v>Bank</v>
       </c>
+      <c r="M127">
+        <v>0</v>
+      </c>
+      <c r="N127" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -5226,6 +5982,12 @@
       <c r="L128" t="str">
         <v>Bank</v>
       </c>
+      <c r="M128">
+        <v>2</v>
+      </c>
+      <c r="N128" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
@@ -5264,6 +6026,12 @@
       <c r="L129" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M129">
+        <v>0</v>
+      </c>
+      <c r="N129" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
@@ -5302,6 +6070,12 @@
       <c r="L130" t="str">
         <v>Bank</v>
       </c>
+      <c r="M130">
+        <v>0</v>
+      </c>
+      <c r="N130" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
@@ -5334,6 +6108,12 @@
       <c r="L131" t="str">
         <v>Bank</v>
       </c>
+      <c r="M131">
+        <v>0</v>
+      </c>
+      <c r="N131" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
@@ -5372,6 +6152,12 @@
       <c r="L132" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M132">
+        <v>0</v>
+      </c>
+      <c r="N132" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
@@ -5410,6 +6196,12 @@
       <c r="L133" t="str">
         <v>Bank</v>
       </c>
+      <c r="M133">
+        <v>2</v>
+      </c>
+      <c r="N133" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -5448,6 +6240,12 @@
       <c r="L134" t="str">
         <v>Bank</v>
       </c>
+      <c r="M134">
+        <v>0</v>
+      </c>
+      <c r="N134" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
@@ -5486,6 +6284,12 @@
       <c r="L135" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M135">
+        <v>0</v>
+      </c>
+      <c r="N135" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
@@ -5524,6 +6328,12 @@
       <c r="L136" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M136">
+        <v>2</v>
+      </c>
+      <c r="N136" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
@@ -5562,6 +6372,12 @@
       <c r="L137" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M137">
+        <v>4</v>
+      </c>
+      <c r="N137" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
@@ -5600,6 +6416,12 @@
       <c r="L138" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M138">
+        <v>20</v>
+      </c>
+      <c r="N138" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
@@ -5638,6 +6460,12 @@
       <c r="L139" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M139">
+        <v>10</v>
+      </c>
+      <c r="N139" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
@@ -5676,6 +6504,12 @@
       <c r="L140" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M140">
+        <v>4</v>
+      </c>
+      <c r="N140" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
@@ -5714,6 +6548,12 @@
       <c r="L141" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M141">
+        <v>2</v>
+      </c>
+      <c r="N141" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
@@ -5752,6 +6592,12 @@
       <c r="L142" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M142">
+        <v>8</v>
+      </c>
+      <c r="N142" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
@@ -5790,6 +6636,12 @@
       <c r="L143" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M143">
+        <v>17</v>
+      </c>
+      <c r="N143" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
@@ -5828,6 +6680,12 @@
       <c r="L144" t="str">
         <v>Bank</v>
       </c>
+      <c r="M144">
+        <v>0</v>
+      </c>
+      <c r="N144" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
@@ -5866,6 +6724,12 @@
       <c r="L145" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M145">
+        <v>6</v>
+      </c>
+      <c r="N145" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
@@ -5904,6 +6768,12 @@
       <c r="L146" t="str">
         <v>Bank</v>
       </c>
+      <c r="M146">
+        <v>0</v>
+      </c>
+      <c r="N146" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
@@ -5942,6 +6812,12 @@
       <c r="L147" t="str">
         <v>Bank</v>
       </c>
+      <c r="M147">
+        <v>2</v>
+      </c>
+      <c r="N147" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
@@ -5980,6 +6856,12 @@
       <c r="L148" t="str">
         <v>Bank</v>
       </c>
+      <c r="M148">
+        <v>2</v>
+      </c>
+      <c r="N148" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
@@ -6018,6 +6900,12 @@
       <c r="L149" t="str">
         <v>Bank</v>
       </c>
+      <c r="M149">
+        <v>0</v>
+      </c>
+      <c r="N149" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
@@ -6056,6 +6944,12 @@
       <c r="L150" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M150">
+        <v>0</v>
+      </c>
+      <c r="N150" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
@@ -6094,6 +6988,12 @@
       <c r="L151" t="str">
         <v>Bank</v>
       </c>
+      <c r="M151">
+        <v>0</v>
+      </c>
+      <c r="N151" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
@@ -6132,6 +7032,12 @@
       <c r="L152" t="str">
         <v>Bank</v>
       </c>
+      <c r="M152">
+        <v>0</v>
+      </c>
+      <c r="N152" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
@@ -6170,6 +7076,12 @@
       <c r="L153" t="str">
         <v>Bank</v>
       </c>
+      <c r="M153">
+        <v>0</v>
+      </c>
+      <c r="N153" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
@@ -6208,6 +7120,12 @@
       <c r="L154" t="str">
         <v>Bank</v>
       </c>
+      <c r="M154">
+        <v>0</v>
+      </c>
+      <c r="N154" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
@@ -6246,6 +7164,12 @@
       <c r="L155" t="str">
         <v>Bank</v>
       </c>
+      <c r="M155">
+        <v>0</v>
+      </c>
+      <c r="N155" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
@@ -6284,6 +7208,12 @@
       <c r="L156" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M156">
+        <v>4</v>
+      </c>
+      <c r="N156" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
@@ -6322,6 +7252,12 @@
       <c r="L157" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M157">
+        <v>-6</v>
+      </c>
+      <c r="N157" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
@@ -6360,6 +7296,12 @@
       <c r="L158" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M158">
+        <v>6</v>
+      </c>
+      <c r="N158" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
@@ -6398,6 +7340,12 @@
       <c r="L159" t="str">
         <v>Bank</v>
       </c>
+      <c r="M159">
+        <v>13</v>
+      </c>
+      <c r="N159" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
@@ -6436,6 +7384,12 @@
       <c r="L160" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M160">
+        <v>4</v>
+      </c>
+      <c r="N160" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
@@ -6474,6 +7428,12 @@
       <c r="L161" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M161">
+        <v>4</v>
+      </c>
+      <c r="N161" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
@@ -6512,6 +7472,12 @@
       <c r="L162" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M162">
+        <v>0</v>
+      </c>
+      <c r="N162" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
@@ -6550,6 +7516,12 @@
       <c r="L163" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M163">
+        <v>10</v>
+      </c>
+      <c r="N163" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
@@ -6588,6 +7560,12 @@
       <c r="L164" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M164">
+        <v>-4</v>
+      </c>
+      <c r="N164" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
@@ -6626,6 +7604,12 @@
       <c r="L165" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M165">
+        <v>11</v>
+      </c>
+      <c r="N165" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
@@ -6664,6 +7648,12 @@
       <c r="L166" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M166">
+        <v>0</v>
+      </c>
+      <c r="N166" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
@@ -6702,6 +7692,12 @@
       <c r="L167" t="str">
         <v>Bank</v>
       </c>
+      <c r="M167">
+        <v>2</v>
+      </c>
+      <c r="N167" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
@@ -6740,6 +7736,12 @@
       <c r="L168" t="str">
         <v>Bank</v>
       </c>
+      <c r="M168">
+        <v>0</v>
+      </c>
+      <c r="N168" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
@@ -6778,6 +7780,12 @@
       <c r="L169" t="str">
         <v>Bank</v>
       </c>
+      <c r="M169">
+        <v>0</v>
+      </c>
+      <c r="N169" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
@@ -6816,6 +7824,12 @@
       <c r="L170" t="str">
         <v>Bank</v>
       </c>
+      <c r="M170">
+        <v>2</v>
+      </c>
+      <c r="N170" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
@@ -6854,6 +7868,12 @@
       <c r="L171" t="str">
         <v>Bank</v>
       </c>
+      <c r="M171">
+        <v>0</v>
+      </c>
+      <c r="N171" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
@@ -6892,6 +7912,12 @@
       <c r="L172" t="str">
         <v>Bank</v>
       </c>
+      <c r="M172">
+        <v>0</v>
+      </c>
+      <c r="N172" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
@@ -6930,6 +7956,12 @@
       <c r="L173" t="str">
         <v>Bank</v>
       </c>
+      <c r="M173">
+        <v>0</v>
+      </c>
+      <c r="N173" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
@@ -6968,6 +8000,12 @@
       <c r="L174" t="str">
         <v>Bank</v>
       </c>
+      <c r="M174">
+        <v>0</v>
+      </c>
+      <c r="N174" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
@@ -7006,6 +8044,12 @@
       <c r="L175" t="str">
         <v>Bank</v>
       </c>
+      <c r="M175">
+        <v>0</v>
+      </c>
+      <c r="N175" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
@@ -7044,6 +8088,12 @@
       <c r="L176" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M176">
+        <v>14</v>
+      </c>
+      <c r="N176" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
@@ -7082,6 +8132,12 @@
       <c r="L177" t="str">
         <v>Bank</v>
       </c>
+      <c r="M177">
+        <v>0</v>
+      </c>
+      <c r="N177" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
@@ -7120,6 +8176,12 @@
       <c r="L178" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M178">
+        <v>8</v>
+      </c>
+      <c r="N178" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
@@ -7158,6 +8220,12 @@
       <c r="L179" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M179">
+        <v>0</v>
+      </c>
+      <c r="N179" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
@@ -7196,6 +8264,12 @@
       <c r="L180" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M180">
+        <v>4</v>
+      </c>
+      <c r="N180" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
@@ -7234,6 +8308,12 @@
       <c r="L181" t="str">
         <v>Bank</v>
       </c>
+      <c r="M181">
+        <v>13</v>
+      </c>
+      <c r="N181" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
@@ -7272,6 +8352,12 @@
       <c r="L182" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M182">
+        <v>4</v>
+      </c>
+      <c r="N182" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
@@ -7310,6 +8396,12 @@
       <c r="L183" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M183">
+        <v>6</v>
+      </c>
+      <c r="N183" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
@@ -7348,6 +8440,12 @@
       <c r="L184" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M184">
+        <v>2</v>
+      </c>
+      <c r="N184" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
@@ -7386,6 +8484,12 @@
       <c r="L185" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M185">
+        <v>0</v>
+      </c>
+      <c r="N185" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
@@ -7424,6 +8528,12 @@
       <c r="L186" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M186">
+        <v>4</v>
+      </c>
+      <c r="N186" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
@@ -7462,6 +8572,12 @@
       <c r="L187" t="str">
         <v>Bank</v>
       </c>
+      <c r="M187">
+        <v>0</v>
+      </c>
+      <c r="N187" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
@@ -7500,6 +8616,12 @@
       <c r="L188" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M188">
+        <v>2</v>
+      </c>
+      <c r="N188" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
@@ -7538,6 +8660,12 @@
       <c r="L189" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M189">
+        <v>0</v>
+      </c>
+      <c r="N189" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
@@ -7576,6 +8704,12 @@
       <c r="L190" t="str">
         <v>Bank</v>
       </c>
+      <c r="M190">
+        <v>0</v>
+      </c>
+      <c r="N190" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
@@ -7614,6 +8748,12 @@
       <c r="L191" t="str">
         <v>Bank</v>
       </c>
+      <c r="M191">
+        <v>0</v>
+      </c>
+      <c r="N191" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
@@ -7652,6 +8792,12 @@
       <c r="L192" t="str">
         <v>Bank</v>
       </c>
+      <c r="M192">
+        <v>0</v>
+      </c>
+      <c r="N192" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
@@ -7684,6 +8830,12 @@
       <c r="L193" t="str">
         <v>Bank</v>
       </c>
+      <c r="M193">
+        <v>0</v>
+      </c>
+      <c r="N193" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
@@ -7722,6 +8874,12 @@
       <c r="L194" t="str">
         <v>Bank</v>
       </c>
+      <c r="M194">
+        <v>0</v>
+      </c>
+      <c r="N194" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
@@ -7760,6 +8918,12 @@
       <c r="L195" t="str">
         <v>Bank</v>
       </c>
+      <c r="M195">
+        <v>0</v>
+      </c>
+      <c r="N195" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
@@ -7798,6 +8962,12 @@
       <c r="L196" t="str">
         <v>Bank</v>
       </c>
+      <c r="M196">
+        <v>0</v>
+      </c>
+      <c r="N196" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
@@ -7836,6 +9006,12 @@
       <c r="L197" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M197">
+        <v>2</v>
+      </c>
+      <c r="N197" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
@@ -7868,6 +9044,12 @@
       <c r="L198" t="str">
         <v>Bank</v>
       </c>
+      <c r="M198">
+        <v>0</v>
+      </c>
+      <c r="N198" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
@@ -7906,6 +9088,12 @@
       <c r="L199" t="str">
         <v>Bank</v>
       </c>
+      <c r="M199">
+        <v>0</v>
+      </c>
+      <c r="N199" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
@@ -7944,6 +9132,12 @@
       <c r="L200" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M200">
+        <v>0</v>
+      </c>
+      <c r="N200" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
@@ -7982,6 +9176,12 @@
       <c r="L201" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M201">
+        <v>20</v>
+      </c>
+      <c r="N201" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
@@ -8020,6 +9220,12 @@
       <c r="L202" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M202">
+        <v>2</v>
+      </c>
+      <c r="N202" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
@@ -8058,6 +9264,12 @@
       <c r="L203" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M203">
+        <v>6</v>
+      </c>
+      <c r="N203" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
@@ -8096,6 +9308,12 @@
       <c r="L204" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M204">
+        <v>6</v>
+      </c>
+      <c r="N204" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
@@ -8134,6 +9352,12 @@
       <c r="L205" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M205">
+        <v>0</v>
+      </c>
+      <c r="N205" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
@@ -8172,6 +9396,12 @@
       <c r="L206" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M206">
+        <v>8</v>
+      </c>
+      <c r="N206" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
@@ -8210,6 +9440,12 @@
       <c r="L207" t="str">
         <v>Bank</v>
       </c>
+      <c r="M207">
+        <v>4</v>
+      </c>
+      <c r="N207" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
@@ -8248,6 +9484,12 @@
       <c r="L208" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M208">
+        <v>10</v>
+      </c>
+      <c r="N208" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
@@ -8286,6 +9528,12 @@
       <c r="L209" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M209">
+        <v>4</v>
+      </c>
+      <c r="N209" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
@@ -8324,6 +9572,12 @@
       <c r="L210" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M210">
+        <v>-2</v>
+      </c>
+      <c r="N210" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
@@ -8362,6 +9616,12 @@
       <c r="L211" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M211">
+        <v>0</v>
+      </c>
+      <c r="N211" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
@@ -8400,6 +9660,12 @@
       <c r="L212" t="str">
         <v>Bank</v>
       </c>
+      <c r="M212">
+        <v>2</v>
+      </c>
+      <c r="N212" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
@@ -8438,6 +9704,12 @@
       <c r="L213" t="str">
         <v>Bank</v>
       </c>
+      <c r="M213">
+        <v>2</v>
+      </c>
+      <c r="N213" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
@@ -8476,6 +9748,12 @@
       <c r="L214" t="str">
         <v>Bank</v>
       </c>
+      <c r="M214">
+        <v>0</v>
+      </c>
+      <c r="N214" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
@@ -8514,6 +9792,12 @@
       <c r="L215" t="str">
         <v>Bank</v>
       </c>
+      <c r="M215">
+        <v>6</v>
+      </c>
+      <c r="N215" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
@@ -8552,6 +9836,12 @@
       <c r="L216" t="str">
         <v>Bank</v>
       </c>
+      <c r="M216">
+        <v>2</v>
+      </c>
+      <c r="N216" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
@@ -8590,6 +9880,12 @@
       <c r="L217" t="str">
         <v>Bank</v>
       </c>
+      <c r="M217">
+        <v>0</v>
+      </c>
+      <c r="N217" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
@@ -8628,6 +9924,12 @@
       <c r="L218" t="str">
         <v>Bank</v>
       </c>
+      <c r="M218">
+        <v>0</v>
+      </c>
+      <c r="N218" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
@@ -8666,6 +9968,12 @@
       <c r="L219" t="str">
         <v>Bank</v>
       </c>
+      <c r="M219">
+        <v>0</v>
+      </c>
+      <c r="N219" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
@@ -8704,6 +10012,12 @@
       <c r="L220" t="str">
         <v>Bank</v>
       </c>
+      <c r="M220">
+        <v>0</v>
+      </c>
+      <c r="N220" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
@@ -8742,6 +10056,12 @@
       <c r="L221" t="str">
         <v>Bank</v>
       </c>
+      <c r="M221">
+        <v>0</v>
+      </c>
+      <c r="N221" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
@@ -8780,6 +10100,12 @@
       <c r="L222" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M222">
+        <v>8</v>
+      </c>
+      <c r="N222" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
@@ -8818,6 +10144,12 @@
       <c r="L223" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M223">
+        <v>0</v>
+      </c>
+      <c r="N223" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
@@ -8856,6 +10188,12 @@
       <c r="L224" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M224">
+        <v>6</v>
+      </c>
+      <c r="N224" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
@@ -8894,6 +10232,12 @@
       <c r="L225" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M225">
+        <v>7</v>
+      </c>
+      <c r="N225" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
@@ -8932,6 +10276,12 @@
       <c r="L226" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M226">
+        <v>0</v>
+      </c>
+      <c r="N226" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
@@ -8970,6 +10320,12 @@
       <c r="L227" t="str">
         <v>Bank</v>
       </c>
+      <c r="M227">
+        <v>0</v>
+      </c>
+      <c r="N227" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
@@ -9008,6 +10364,12 @@
       <c r="L228" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M228">
+        <v>8</v>
+      </c>
+      <c r="N228" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
@@ -9046,6 +10408,12 @@
       <c r="L229" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M229">
+        <v>6</v>
+      </c>
+      <c r="N229" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
@@ -9084,6 +10452,12 @@
       <c r="L230" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M230">
+        <v>-2</v>
+      </c>
+      <c r="N230" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
@@ -9122,6 +10496,12 @@
       <c r="L231" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M231">
+        <v>0</v>
+      </c>
+      <c r="N231" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
@@ -9160,6 +10540,12 @@
       <c r="L232" t="str">
         <v>Bank</v>
       </c>
+      <c r="M232">
+        <v>0</v>
+      </c>
+      <c r="N232" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
@@ -9198,6 +10584,12 @@
       <c r="L233" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M233">
+        <v>2</v>
+      </c>
+      <c r="N233" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
@@ -9236,6 +10628,12 @@
       <c r="L234" t="str">
         <v>Bank</v>
       </c>
+      <c r="M234">
+        <v>2</v>
+      </c>
+      <c r="N234" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
@@ -9274,6 +10672,12 @@
       <c r="L235" t="str">
         <v>Bank</v>
       </c>
+      <c r="M235">
+        <v>0</v>
+      </c>
+      <c r="N235" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
@@ -9312,6 +10716,12 @@
       <c r="L236" t="str">
         <v>Bank</v>
       </c>
+      <c r="M236">
+        <v>0</v>
+      </c>
+      <c r="N236" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
@@ -9350,6 +10760,12 @@
       <c r="L237" t="str">
         <v>Bank</v>
       </c>
+      <c r="M237">
+        <v>0</v>
+      </c>
+      <c r="N237" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
@@ -9388,6 +10804,12 @@
       <c r="L238" t="str">
         <v>Bank</v>
       </c>
+      <c r="M238">
+        <v>0</v>
+      </c>
+      <c r="N238" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
@@ -9426,6 +10848,12 @@
       <c r="L239" t="str">
         <v>Bank</v>
       </c>
+      <c r="M239">
+        <v>0</v>
+      </c>
+      <c r="N239" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
@@ -9464,6 +10892,12 @@
       <c r="L240" t="str">
         <v>Bank</v>
       </c>
+      <c r="M240">
+        <v>0</v>
+      </c>
+      <c r="N240" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
@@ -9502,6 +10936,12 @@
       <c r="L241" t="str">
         <v>Bank</v>
       </c>
+      <c r="M241">
+        <v>0</v>
+      </c>
+      <c r="N241" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
@@ -9540,6 +10980,12 @@
       <c r="L242" t="str">
         <v>Startelf</v>
       </c>
+      <c r="M242">
+        <v>2</v>
+      </c>
+      <c r="N242" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
@@ -9576,6 +11022,12 @@
         <v>0</v>
       </c>
       <c r="L243" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="M243">
+        <v>0</v>
+      </c>
+      <c r="N243" t="str">
         <v>Bank</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Spieltag 6 (2026/27): Daten, Kaderseiten und Portal-Tabelle aktualisiert
- Datendateien aus D:\Spreeliga\stand aufgefrischt: saison.xlsx, players-se.csv,
  spieltagspunkte.csv, clientdb.json, historie/manager.json, stats/saison.json,
  neu stats/st6.json, stats/powerverlauf.json.
- Alle 11 manager-*.html und portal.html mit werkstatt\bauen\website.js erzeugt.
- Erzeugt von werkstatt\spieltag.js; im Lauf vom 20.10.2026 brach das git add ab, weil
  beim Zerlegen der git-status-Zeilen ein Zeichen zu viel abgeschnitten wurde. Behoben.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/saison.xlsx
+++ b/saison.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N243"/>
+  <dimension ref="A1:P243"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,6 +442,12 @@
       <c r="N1" t="str">
         <v>ST5 Rolle</v>
       </c>
+      <c r="O1" t="str">
+        <v>ST6 Punkte</v>
+      </c>
+      <c r="P1" t="str">
+        <v>ST6 Rolle</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -486,6 +492,12 @@
       <c r="N2" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O2">
+        <v>6</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -530,6 +542,12 @@
       <c r="N3" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -574,6 +592,12 @@
       <c r="N4" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O4">
+        <v>2</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -618,6 +642,12 @@
       <c r="N5" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O5">
+        <v>2</v>
+      </c>
+      <c r="P5" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -662,6 +692,12 @@
       <c r="N6" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O6">
+        <v>2</v>
+      </c>
+      <c r="P6" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -706,6 +742,12 @@
       <c r="N7" t="str">
         <v>Bank</v>
       </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -750,6 +792,12 @@
       <c r="N8" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O8">
+        <v>2</v>
+      </c>
+      <c r="P8" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -794,6 +842,12 @@
       <c r="N9" t="str">
         <v>Bank</v>
       </c>
+      <c r="O9">
+        <v>2</v>
+      </c>
+      <c r="P9" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -838,6 +892,12 @@
       <c r="N10" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O10">
+        <v>17</v>
+      </c>
+      <c r="P10" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -882,6 +942,12 @@
       <c r="N11" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O11">
+        <v>-2</v>
+      </c>
+      <c r="P11" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -926,6 +992,12 @@
       <c r="N12" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O12">
+        <v>13</v>
+      </c>
+      <c r="P12" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -970,6 +1042,12 @@
       <c r="N13" t="str">
         <v>Bank</v>
       </c>
+      <c r="O13">
+        <v>0</v>
+      </c>
+      <c r="P13" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1014,6 +1092,12 @@
       <c r="N14" t="str">
         <v>Bank</v>
       </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1058,6 +1142,12 @@
       <c r="N15" t="str">
         <v>Bank</v>
       </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1102,6 +1192,12 @@
       <c r="N16" t="str">
         <v>Bank</v>
       </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1146,6 +1242,12 @@
       <c r="N17" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1190,6 +1292,12 @@
       <c r="N18" t="str">
         <v>Bank</v>
       </c>
+      <c r="O18">
+        <v>2</v>
+      </c>
+      <c r="P18" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1234,6 +1342,12 @@
       <c r="N19" t="str">
         <v>Bank</v>
       </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1278,6 +1392,12 @@
       <c r="N20" t="str">
         <v>Bank</v>
       </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1322,6 +1442,12 @@
       <c r="N21" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O21">
+        <v>6</v>
+      </c>
+      <c r="P21" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1366,6 +1492,12 @@
       <c r="N22" t="str">
         <v>Bank</v>
       </c>
+      <c r="O22">
+        <v>2</v>
+      </c>
+      <c r="P22" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1410,6 +1542,12 @@
       <c r="N23" t="str">
         <v>Bank</v>
       </c>
+      <c r="O23">
+        <v>0</v>
+      </c>
+      <c r="P23" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1454,6 +1592,12 @@
       <c r="N24" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O24">
+        <v>17</v>
+      </c>
+      <c r="P24" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1498,6 +1642,12 @@
       <c r="N25" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="P25" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1536,6 +1686,12 @@
       <c r="N26" t="str">
         <v>Bank</v>
       </c>
+      <c r="O26">
+        <v>0</v>
+      </c>
+      <c r="P26" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1580,6 +1736,12 @@
       <c r="N27" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O27">
+        <v>0</v>
+      </c>
+      <c r="P27" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1624,6 +1786,12 @@
       <c r="N28" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O28">
+        <v>0</v>
+      </c>
+      <c r="P28" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1668,6 +1836,12 @@
       <c r="N29" t="str">
         <v>Bank</v>
       </c>
+      <c r="O29">
+        <v>0</v>
+      </c>
+      <c r="P29" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1712,6 +1886,12 @@
       <c r="N30" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O30">
+        <v>6</v>
+      </c>
+      <c r="P30" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1756,6 +1936,12 @@
       <c r="N31" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O31">
+        <v>6</v>
+      </c>
+      <c r="P31" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1800,6 +1986,12 @@
       <c r="N32" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O32">
+        <v>17</v>
+      </c>
+      <c r="P32" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1844,6 +2036,12 @@
       <c r="N33" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O33">
+        <v>21</v>
+      </c>
+      <c r="P33" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1888,6 +2086,12 @@
       <c r="N34" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O34">
+        <v>16</v>
+      </c>
+      <c r="P34" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1932,6 +2136,12 @@
       <c r="N35" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O35">
+        <v>0</v>
+      </c>
+      <c r="P35" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1976,6 +2186,12 @@
       <c r="N36" t="str">
         <v>Bank</v>
       </c>
+      <c r="O36">
+        <v>0</v>
+      </c>
+      <c r="P36" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -2020,6 +2236,12 @@
       <c r="N37" t="str">
         <v>Bank</v>
       </c>
+      <c r="O37">
+        <v>0</v>
+      </c>
+      <c r="P37" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -2064,6 +2286,12 @@
       <c r="N38" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O38">
+        <v>0</v>
+      </c>
+      <c r="P38" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -2108,6 +2336,12 @@
       <c r="N39" t="str">
         <v>Bank</v>
       </c>
+      <c r="O39">
+        <v>2</v>
+      </c>
+      <c r="P39" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -2152,6 +2386,12 @@
       <c r="N40" t="str">
         <v>Bank</v>
       </c>
+      <c r="O40">
+        <v>0</v>
+      </c>
+      <c r="P40" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -2196,6 +2436,12 @@
       <c r="N41" t="str">
         <v>Bank</v>
       </c>
+      <c r="O41">
+        <v>2</v>
+      </c>
+      <c r="P41" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -2240,6 +2486,12 @@
       <c r="N42" t="str">
         <v>Bank</v>
       </c>
+      <c r="O42">
+        <v>0</v>
+      </c>
+      <c r="P42" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -2278,6 +2530,12 @@
       <c r="N43" t="str">
         <v>Bank</v>
       </c>
+      <c r="O43">
+        <v>0</v>
+      </c>
+      <c r="P43" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -2322,6 +2580,12 @@
       <c r="N44" t="str">
         <v>Bank</v>
       </c>
+      <c r="O44">
+        <v>0</v>
+      </c>
+      <c r="P44" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -2366,6 +2630,12 @@
       <c r="N45" t="str">
         <v>Bank</v>
       </c>
+      <c r="O45">
+        <v>0</v>
+      </c>
+      <c r="P45" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -2410,6 +2680,12 @@
       <c r="N46" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O46">
+        <v>6</v>
+      </c>
+      <c r="P46" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -2454,6 +2730,12 @@
       <c r="N47" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O47">
+        <v>12</v>
+      </c>
+      <c r="P47" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -2498,6 +2780,12 @@
       <c r="N48" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O48">
+        <v>4</v>
+      </c>
+      <c r="P48" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -2542,6 +2830,12 @@
       <c r="N49" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O49">
+        <v>2</v>
+      </c>
+      <c r="P49" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -2586,6 +2880,12 @@
       <c r="N50" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O50">
+        <v>2</v>
+      </c>
+      <c r="P50" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -2630,6 +2930,12 @@
       <c r="N51" t="str">
         <v>Bank</v>
       </c>
+      <c r="O51">
+        <v>0</v>
+      </c>
+      <c r="P51" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -2674,6 +2980,12 @@
       <c r="N52" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O52">
+        <v>10</v>
+      </c>
+      <c r="P52" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -2718,6 +3030,12 @@
       <c r="N53" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O53">
+        <v>2</v>
+      </c>
+      <c r="P53" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -2762,6 +3080,12 @@
       <c r="N54" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O54">
+        <v>17</v>
+      </c>
+      <c r="P54" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -2806,6 +3130,12 @@
       <c r="N55" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O55">
+        <v>13</v>
+      </c>
+      <c r="P55" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2850,6 +3180,12 @@
       <c r="N56" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O56">
+        <v>0</v>
+      </c>
+      <c r="P56" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2894,6 +3230,12 @@
       <c r="N57" t="str">
         <v>Bank</v>
       </c>
+      <c r="O57">
+        <v>0</v>
+      </c>
+      <c r="P57" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -2938,6 +3280,12 @@
       <c r="N58" t="str">
         <v>Bank</v>
       </c>
+      <c r="O58">
+        <v>0</v>
+      </c>
+      <c r="P58" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2982,6 +3330,12 @@
       <c r="N59" t="str">
         <v>Bank</v>
       </c>
+      <c r="O59">
+        <v>0</v>
+      </c>
+      <c r="P59" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -3026,6 +3380,12 @@
       <c r="N60" t="str">
         <v>Bank</v>
       </c>
+      <c r="O60">
+        <v>4</v>
+      </c>
+      <c r="P60" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -3070,6 +3430,12 @@
       <c r="N61" t="str">
         <v>Bank</v>
       </c>
+      <c r="O61">
+        <v>2</v>
+      </c>
+      <c r="P61" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -3114,6 +3480,12 @@
       <c r="N62" t="str">
         <v>Bank</v>
       </c>
+      <c r="O62">
+        <v>2</v>
+      </c>
+      <c r="P62" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -3158,6 +3530,12 @@
       <c r="N63" t="str">
         <v>Bank</v>
       </c>
+      <c r="O63">
+        <v>0</v>
+      </c>
+      <c r="P63" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -3202,6 +3580,12 @@
       <c r="N64" t="str">
         <v>Bank</v>
       </c>
+      <c r="O64">
+        <v>0</v>
+      </c>
+      <c r="P64" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -3246,6 +3630,12 @@
       <c r="N65" t="str">
         <v>Bank</v>
       </c>
+      <c r="O65">
+        <v>0</v>
+      </c>
+      <c r="P65" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -3290,6 +3680,12 @@
       <c r="N66" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O66">
+        <v>6</v>
+      </c>
+      <c r="P66" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -3334,6 +3730,12 @@
       <c r="N67" t="str">
         <v>Bank</v>
       </c>
+      <c r="O67">
+        <v>2</v>
+      </c>
+      <c r="P67" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -3378,6 +3780,12 @@
       <c r="N68" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O68">
+        <v>17</v>
+      </c>
+      <c r="P68" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -3422,6 +3830,12 @@
       <c r="N69" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O69">
+        <v>2</v>
+      </c>
+      <c r="P69" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -3466,6 +3880,12 @@
       <c r="N70" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O70">
+        <v>2</v>
+      </c>
+      <c r="P70" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -3510,6 +3930,12 @@
       <c r="N71" t="str">
         <v>Bank</v>
       </c>
+      <c r="O71">
+        <v>6</v>
+      </c>
+      <c r="P71" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -3554,6 +3980,12 @@
       <c r="N72" t="str">
         <v>Bank</v>
       </c>
+      <c r="O72">
+        <v>-2</v>
+      </c>
+      <c r="P72" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -3598,6 +4030,12 @@
       <c r="N73" t="str">
         <v>Bank</v>
       </c>
+      <c r="O73">
+        <v>2</v>
+      </c>
+      <c r="P73" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -3642,6 +4080,12 @@
       <c r="N74" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O74">
+        <v>0</v>
+      </c>
+      <c r="P74" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -3686,6 +4130,12 @@
       <c r="N75" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O75">
+        <v>2</v>
+      </c>
+      <c r="P75" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -3730,6 +4180,12 @@
       <c r="N76" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O76">
+        <v>13</v>
+      </c>
+      <c r="P76" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -3774,6 +4230,12 @@
       <c r="N77" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O77">
+        <v>4</v>
+      </c>
+      <c r="P77" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -3818,6 +4280,12 @@
       <c r="N78" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O78">
+        <v>17</v>
+      </c>
+      <c r="P78" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -3862,6 +4330,12 @@
       <c r="N79" t="str">
         <v>Bank</v>
       </c>
+      <c r="O79">
+        <v>0</v>
+      </c>
+      <c r="P79" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -3906,6 +4380,12 @@
       <c r="N80" t="str">
         <v>Bank</v>
       </c>
+      <c r="O80">
+        <v>0</v>
+      </c>
+      <c r="P80" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -3950,6 +4430,12 @@
       <c r="N81" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O81">
+        <v>4</v>
+      </c>
+      <c r="P81" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -3988,6 +4474,12 @@
       <c r="N82" t="str">
         <v>Bank</v>
       </c>
+      <c r="O82">
+        <v>0</v>
+      </c>
+      <c r="P82" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -4032,6 +4524,12 @@
       <c r="N83" t="str">
         <v>Bank</v>
       </c>
+      <c r="O83">
+        <v>0</v>
+      </c>
+      <c r="P83" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -4076,6 +4574,12 @@
       <c r="N84" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O84">
+        <v>0</v>
+      </c>
+      <c r="P84" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -4120,6 +4624,12 @@
       <c r="N85" t="str">
         <v>Bank</v>
       </c>
+      <c r="O85">
+        <v>2</v>
+      </c>
+      <c r="P85" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -4164,6 +4674,12 @@
       <c r="N86" t="str">
         <v>Bank</v>
       </c>
+      <c r="O86">
+        <v>0</v>
+      </c>
+      <c r="P86" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -4208,6 +4724,12 @@
       <c r="N87" t="str">
         <v>Bank</v>
       </c>
+      <c r="O87">
+        <v>2</v>
+      </c>
+      <c r="P87" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -4252,6 +4774,12 @@
       <c r="N88" t="str">
         <v>Bank</v>
       </c>
+      <c r="O88">
+        <v>0</v>
+      </c>
+      <c r="P88" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -4296,6 +4824,12 @@
       <c r="N89" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O89">
+        <v>6</v>
+      </c>
+      <c r="P89" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -4340,6 +4874,12 @@
       <c r="N90" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O90">
+        <v>8</v>
+      </c>
+      <c r="P90" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -4384,6 +4924,12 @@
       <c r="N91" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O91">
+        <v>4</v>
+      </c>
+      <c r="P91" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -4428,6 +4974,12 @@
       <c r="N92" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O92">
+        <v>12</v>
+      </c>
+      <c r="P92" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -4472,6 +5024,12 @@
       <c r="N93" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O93">
+        <v>2</v>
+      </c>
+      <c r="P93" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -4516,6 +5074,12 @@
       <c r="N94" t="str">
         <v>Bank</v>
       </c>
+      <c r="O94">
+        <v>0</v>
+      </c>
+      <c r="P94" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -4560,6 +5124,12 @@
       <c r="N95" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O95">
+        <v>6</v>
+      </c>
+      <c r="P95" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -4604,6 +5174,12 @@
       <c r="N96" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O96">
+        <v>16</v>
+      </c>
+      <c r="P96" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -4648,6 +5224,12 @@
       <c r="N97" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O97">
+        <v>2</v>
+      </c>
+      <c r="P97" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -4692,6 +5274,12 @@
       <c r="N98" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O98">
+        <v>4</v>
+      </c>
+      <c r="P98" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -4736,6 +5324,12 @@
       <c r="N99" t="str">
         <v>Bank</v>
       </c>
+      <c r="O99">
+        <v>-2</v>
+      </c>
+      <c r="P99" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -4780,6 +5374,12 @@
       <c r="N100" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O100">
+        <v>4</v>
+      </c>
+      <c r="P100" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -4824,6 +5424,12 @@
       <c r="N101" t="str">
         <v>Bank</v>
       </c>
+      <c r="O101">
+        <v>2</v>
+      </c>
+      <c r="P101" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -4868,6 +5474,12 @@
       <c r="N102" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O102">
+        <v>9</v>
+      </c>
+      <c r="P102" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -4912,6 +5524,12 @@
       <c r="N103" t="str">
         <v>Bank</v>
       </c>
+      <c r="O103">
+        <v>2</v>
+      </c>
+      <c r="P103" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -4950,6 +5568,12 @@
       <c r="N104" t="str">
         <v>Bank</v>
       </c>
+      <c r="O104">
+        <v>0</v>
+      </c>
+      <c r="P104" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -4994,6 +5618,12 @@
       <c r="N105" t="str">
         <v>Bank</v>
       </c>
+      <c r="O105">
+        <v>0</v>
+      </c>
+      <c r="P105" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -5038,6 +5668,12 @@
       <c r="N106" t="str">
         <v>Bank</v>
       </c>
+      <c r="O106">
+        <v>0</v>
+      </c>
+      <c r="P106" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -5076,6 +5712,12 @@
       <c r="N107" t="str">
         <v>Bank</v>
       </c>
+      <c r="O107">
+        <v>0</v>
+      </c>
+      <c r="P107" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -5120,6 +5762,12 @@
       <c r="N108" t="str">
         <v>Bank</v>
       </c>
+      <c r="O108">
+        <v>0</v>
+      </c>
+      <c r="P108" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -5164,6 +5812,12 @@
       <c r="N109" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O109">
+        <v>2</v>
+      </c>
+      <c r="P109" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -5208,6 +5862,12 @@
       <c r="N110" t="str">
         <v>Bank</v>
       </c>
+      <c r="O110">
+        <v>0</v>
+      </c>
+      <c r="P110" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -5246,6 +5906,12 @@
       <c r="N111" t="str">
         <v>Bank</v>
       </c>
+      <c r="O111">
+        <v>0</v>
+      </c>
+      <c r="P111" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -5290,6 +5956,12 @@
       <c r="N112" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O112">
+        <v>4</v>
+      </c>
+      <c r="P112" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -5334,6 +6006,12 @@
       <c r="N113" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O113">
+        <v>8</v>
+      </c>
+      <c r="P113" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -5378,6 +6056,12 @@
       <c r="N114" t="str">
         <v>Bank</v>
       </c>
+      <c r="O114">
+        <v>6</v>
+      </c>
+      <c r="P114" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -5422,6 +6106,12 @@
       <c r="N115" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O115">
+        <v>6</v>
+      </c>
+      <c r="P115" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -5466,6 +6156,12 @@
       <c r="N116" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O116">
+        <v>6</v>
+      </c>
+      <c r="P116" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -5510,6 +6206,12 @@
       <c r="N117" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O117">
+        <v>21</v>
+      </c>
+      <c r="P117" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -5554,6 +6256,12 @@
       <c r="N118" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O118">
+        <v>2</v>
+      </c>
+      <c r="P118" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -5598,6 +6306,12 @@
       <c r="N119" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O119">
+        <v>0</v>
+      </c>
+      <c r="P119" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -5642,6 +6356,12 @@
       <c r="N120" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O120">
+        <v>4</v>
+      </c>
+      <c r="P120" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -5686,6 +6406,12 @@
       <c r="N121" t="str">
         <v>Bank</v>
       </c>
+      <c r="O121">
+        <v>0</v>
+      </c>
+      <c r="P121" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -5730,6 +6456,12 @@
       <c r="N122" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O122">
+        <v>21</v>
+      </c>
+      <c r="P122" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -5774,6 +6506,12 @@
       <c r="N123" t="str">
         <v>Bank</v>
       </c>
+      <c r="O123">
+        <v>0</v>
+      </c>
+      <c r="P123" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -5818,6 +6556,12 @@
       <c r="N124" t="str">
         <v>Bank</v>
       </c>
+      <c r="O124">
+        <v>0</v>
+      </c>
+      <c r="P124" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -5862,6 +6606,12 @@
       <c r="N125" t="str">
         <v>Bank</v>
       </c>
+      <c r="O125">
+        <v>0</v>
+      </c>
+      <c r="P125" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -5900,6 +6650,12 @@
       <c r="N126" t="str">
         <v>Bank</v>
       </c>
+      <c r="O126">
+        <v>0</v>
+      </c>
+      <c r="P126" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -5944,6 +6700,12 @@
       <c r="N127" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O127">
+        <v>0</v>
+      </c>
+      <c r="P127" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -5988,6 +6750,12 @@
       <c r="N128" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O128">
+        <v>4</v>
+      </c>
+      <c r="P128" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
@@ -6032,6 +6800,12 @@
       <c r="N129" t="str">
         <v>Bank</v>
       </c>
+      <c r="O129">
+        <v>2</v>
+      </c>
+      <c r="P129" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
@@ -6076,6 +6850,12 @@
       <c r="N130" t="str">
         <v>Bank</v>
       </c>
+      <c r="O130">
+        <v>0</v>
+      </c>
+      <c r="P130" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
@@ -6114,6 +6894,12 @@
       <c r="N131" t="str">
         <v>Bank</v>
       </c>
+      <c r="O131">
+        <v>0</v>
+      </c>
+      <c r="P131" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
@@ -6158,6 +6944,12 @@
       <c r="N132" t="str">
         <v>Bank</v>
       </c>
+      <c r="O132">
+        <v>0</v>
+      </c>
+      <c r="P132" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
@@ -6202,6 +6994,12 @@
       <c r="N133" t="str">
         <v>Bank</v>
       </c>
+      <c r="O133">
+        <v>0</v>
+      </c>
+      <c r="P133" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -6246,6 +7044,12 @@
       <c r="N134" t="str">
         <v>Bank</v>
       </c>
+      <c r="O134">
+        <v>0</v>
+      </c>
+      <c r="P134" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
@@ -6290,6 +7094,12 @@
       <c r="N135" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O135">
+        <v>0</v>
+      </c>
+      <c r="P135" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
@@ -6334,6 +7144,12 @@
       <c r="N136" t="str">
         <v>Bank</v>
       </c>
+      <c r="O136">
+        <v>6</v>
+      </c>
+      <c r="P136" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
@@ -6378,6 +7194,12 @@
       <c r="N137" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O137">
+        <v>6</v>
+      </c>
+      <c r="P137" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
@@ -6422,6 +7244,12 @@
       <c r="N138" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O138">
+        <v>8</v>
+      </c>
+      <c r="P138" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
@@ -6466,6 +7294,12 @@
       <c r="N139" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O139">
+        <v>0</v>
+      </c>
+      <c r="P139" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
@@ -6510,6 +7344,12 @@
       <c r="N140" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O140">
+        <v>0</v>
+      </c>
+      <c r="P140" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
@@ -6554,6 +7394,12 @@
       <c r="N141" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O141">
+        <v>10</v>
+      </c>
+      <c r="P141" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
@@ -6598,6 +7444,12 @@
       <c r="N142" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O142">
+        <v>2</v>
+      </c>
+      <c r="P142" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
@@ -6642,6 +7494,12 @@
       <c r="N143" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O143">
+        <v>21</v>
+      </c>
+      <c r="P143" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
@@ -6686,6 +7544,12 @@
       <c r="N144" t="str">
         <v>Bank</v>
       </c>
+      <c r="O144">
+        <v>0</v>
+      </c>
+      <c r="P144" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
@@ -6730,6 +7594,12 @@
       <c r="N145" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O145">
+        <v>8</v>
+      </c>
+      <c r="P145" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
@@ -6774,6 +7644,12 @@
       <c r="N146" t="str">
         <v>Bank</v>
       </c>
+      <c r="O146">
+        <v>0</v>
+      </c>
+      <c r="P146" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
@@ -6818,6 +7694,12 @@
       <c r="N147" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O147">
+        <v>4</v>
+      </c>
+      <c r="P147" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
@@ -6862,6 +7744,12 @@
       <c r="N148" t="str">
         <v>Bank</v>
       </c>
+      <c r="O148">
+        <v>0</v>
+      </c>
+      <c r="P148" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
@@ -6906,6 +7794,12 @@
       <c r="N149" t="str">
         <v>Bank</v>
       </c>
+      <c r="O149">
+        <v>0</v>
+      </c>
+      <c r="P149" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
@@ -6950,6 +7844,12 @@
       <c r="N150" t="str">
         <v>Bank</v>
       </c>
+      <c r="O150">
+        <v>0</v>
+      </c>
+      <c r="P150" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
@@ -6994,6 +7894,12 @@
       <c r="N151" t="str">
         <v>Bank</v>
       </c>
+      <c r="O151">
+        <v>2</v>
+      </c>
+      <c r="P151" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
@@ -7038,6 +7944,12 @@
       <c r="N152" t="str">
         <v>Bank</v>
       </c>
+      <c r="O152">
+        <v>2</v>
+      </c>
+      <c r="P152" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
@@ -7082,6 +7994,12 @@
       <c r="N153" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O153">
+        <v>2</v>
+      </c>
+      <c r="P153" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
@@ -7126,6 +8044,12 @@
       <c r="N154" t="str">
         <v>Bank</v>
       </c>
+      <c r="O154">
+        <v>0</v>
+      </c>
+      <c r="P154" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
@@ -7170,6 +8094,12 @@
       <c r="N155" t="str">
         <v>Bank</v>
       </c>
+      <c r="O155">
+        <v>0</v>
+      </c>
+      <c r="P155" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
@@ -7214,6 +8144,12 @@
       <c r="N156" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O156">
+        <v>6</v>
+      </c>
+      <c r="P156" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
@@ -7258,6 +8194,12 @@
       <c r="N157" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O157">
+        <v>6</v>
+      </c>
+      <c r="P157" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
@@ -7302,6 +8244,12 @@
       <c r="N158" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O158">
+        <v>2</v>
+      </c>
+      <c r="P158" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
@@ -7346,6 +8294,12 @@
       <c r="N159" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O159">
+        <v>8</v>
+      </c>
+      <c r="P159" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
@@ -7390,6 +8344,12 @@
       <c r="N160" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O160">
+        <v>2</v>
+      </c>
+      <c r="P160" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
@@ -7434,6 +8394,12 @@
       <c r="N161" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O161">
+        <v>2</v>
+      </c>
+      <c r="P161" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
@@ -7478,6 +8444,12 @@
       <c r="N162" t="str">
         <v>Bank</v>
       </c>
+      <c r="O162">
+        <v>-2</v>
+      </c>
+      <c r="P162" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
@@ -7522,6 +8494,12 @@
       <c r="N163" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O163">
+        <v>0</v>
+      </c>
+      <c r="P163" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
@@ -7566,6 +8544,12 @@
       <c r="N164" t="str">
         <v>Bank</v>
       </c>
+      <c r="O164">
+        <v>14</v>
+      </c>
+      <c r="P164" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
@@ -7610,6 +8594,12 @@
       <c r="N165" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O165">
+        <v>16</v>
+      </c>
+      <c r="P165" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
@@ -7654,6 +8644,12 @@
       <c r="N166" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O166">
+        <v>13</v>
+      </c>
+      <c r="P166" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
@@ -7698,6 +8694,12 @@
       <c r="N167" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O167">
+        <v>2</v>
+      </c>
+      <c r="P167" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
@@ -7742,6 +8744,12 @@
       <c r="N168" t="str">
         <v>Bank</v>
       </c>
+      <c r="O168">
+        <v>0</v>
+      </c>
+      <c r="P168" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
@@ -7786,6 +8794,12 @@
       <c r="N169" t="str">
         <v>Bank</v>
       </c>
+      <c r="O169">
+        <v>0</v>
+      </c>
+      <c r="P169" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
@@ -7830,6 +8844,12 @@
       <c r="N170" t="str">
         <v>Bank</v>
       </c>
+      <c r="O170">
+        <v>0</v>
+      </c>
+      <c r="P170" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
@@ -7874,6 +8894,12 @@
       <c r="N171" t="str">
         <v>Bank</v>
       </c>
+      <c r="O171">
+        <v>2</v>
+      </c>
+      <c r="P171" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
@@ -7918,6 +8944,12 @@
       <c r="N172" t="str">
         <v>Bank</v>
       </c>
+      <c r="O172">
+        <v>0</v>
+      </c>
+      <c r="P172" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
@@ -7962,6 +8994,12 @@
       <c r="N173" t="str">
         <v>Bank</v>
       </c>
+      <c r="O173">
+        <v>0</v>
+      </c>
+      <c r="P173" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
@@ -8006,6 +9044,12 @@
       <c r="N174" t="str">
         <v>Bank</v>
       </c>
+      <c r="O174">
+        <v>0</v>
+      </c>
+      <c r="P174" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
@@ -8050,6 +9094,12 @@
       <c r="N175" t="str">
         <v>Bank</v>
       </c>
+      <c r="O175">
+        <v>0</v>
+      </c>
+      <c r="P175" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
@@ -8094,6 +9144,12 @@
       <c r="N176" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O176">
+        <v>6</v>
+      </c>
+      <c r="P176" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
@@ -8138,6 +9194,12 @@
       <c r="N177" t="str">
         <v>Bank</v>
       </c>
+      <c r="O177">
+        <v>0</v>
+      </c>
+      <c r="P177" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
@@ -8182,6 +9244,12 @@
       <c r="N178" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O178">
+        <v>6</v>
+      </c>
+      <c r="P178" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
@@ -8226,6 +9294,12 @@
       <c r="N179" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O179">
+        <v>10</v>
+      </c>
+      <c r="P179" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
@@ -8270,6 +9344,12 @@
       <c r="N180" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O180">
+        <v>6</v>
+      </c>
+      <c r="P180" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
@@ -8314,6 +9394,12 @@
       <c r="N181" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O181">
+        <v>8</v>
+      </c>
+      <c r="P181" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
@@ -8358,6 +9444,12 @@
       <c r="N182" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O182">
+        <v>4</v>
+      </c>
+      <c r="P182" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
@@ -8402,6 +9494,12 @@
       <c r="N183" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O183">
+        <v>21</v>
+      </c>
+      <c r="P183" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
@@ -8446,6 +9544,12 @@
       <c r="N184" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O184">
+        <v>2</v>
+      </c>
+      <c r="P184" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
@@ -8490,6 +9594,12 @@
       <c r="N185" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O185">
+        <v>-2</v>
+      </c>
+      <c r="P185" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
@@ -8534,6 +9644,12 @@
       <c r="N186" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O186">
+        <v>4</v>
+      </c>
+      <c r="P186" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
@@ -8578,6 +9694,12 @@
       <c r="N187" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O187">
+        <v>0</v>
+      </c>
+      <c r="P187" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
@@ -8622,6 +9744,12 @@
       <c r="N188" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O188">
+        <v>2</v>
+      </c>
+      <c r="P188" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
@@ -8666,6 +9794,12 @@
       <c r="N189" t="str">
         <v>Bank</v>
       </c>
+      <c r="O189">
+        <v>0</v>
+      </c>
+      <c r="P189" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
@@ -8710,6 +9844,12 @@
       <c r="N190" t="str">
         <v>Bank</v>
       </c>
+      <c r="O190">
+        <v>0</v>
+      </c>
+      <c r="P190" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
@@ -8754,6 +9894,12 @@
       <c r="N191" t="str">
         <v>Bank</v>
       </c>
+      <c r="O191">
+        <v>0</v>
+      </c>
+      <c r="P191" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
@@ -8798,6 +9944,12 @@
       <c r="N192" t="str">
         <v>Bank</v>
       </c>
+      <c r="O192">
+        <v>0</v>
+      </c>
+      <c r="P192" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
@@ -8836,6 +9988,12 @@
       <c r="N193" t="str">
         <v>Bank</v>
       </c>
+      <c r="O193">
+        <v>0</v>
+      </c>
+      <c r="P193" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
@@ -8880,6 +10038,12 @@
       <c r="N194" t="str">
         <v>Bank</v>
       </c>
+      <c r="O194">
+        <v>0</v>
+      </c>
+      <c r="P194" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
@@ -8924,6 +10088,12 @@
       <c r="N195" t="str">
         <v>Bank</v>
       </c>
+      <c r="O195">
+        <v>0</v>
+      </c>
+      <c r="P195" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
@@ -8968,6 +10138,12 @@
       <c r="N196" t="str">
         <v>Bank</v>
       </c>
+      <c r="O196">
+        <v>0</v>
+      </c>
+      <c r="P196" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
@@ -9012,6 +10188,12 @@
       <c r="N197" t="str">
         <v>Bank</v>
       </c>
+      <c r="O197">
+        <v>0</v>
+      </c>
+      <c r="P197" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
@@ -9050,6 +10232,12 @@
       <c r="N198" t="str">
         <v>Bank</v>
       </c>
+      <c r="O198">
+        <v>0</v>
+      </c>
+      <c r="P198" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
@@ -9094,6 +10282,12 @@
       <c r="N199" t="str">
         <v>Bank</v>
       </c>
+      <c r="O199">
+        <v>0</v>
+      </c>
+      <c r="P199" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
@@ -9138,6 +10332,12 @@
       <c r="N200" t="str">
         <v>Bank</v>
       </c>
+      <c r="O200">
+        <v>0</v>
+      </c>
+      <c r="P200" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
@@ -9182,6 +10382,12 @@
       <c r="N201" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O201">
+        <v>8</v>
+      </c>
+      <c r="P201" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
@@ -9226,6 +10432,12 @@
       <c r="N202" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O202">
+        <v>2</v>
+      </c>
+      <c r="P202" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
@@ -9270,6 +10482,12 @@
       <c r="N203" t="str">
         <v>Bank</v>
       </c>
+      <c r="O203">
+        <v>6</v>
+      </c>
+      <c r="P203" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
@@ -9314,6 +10532,12 @@
       <c r="N204" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O204">
+        <v>21</v>
+      </c>
+      <c r="P204" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
@@ -9358,6 +10582,12 @@
       <c r="N205" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O205">
+        <v>0</v>
+      </c>
+      <c r="P205" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
@@ -9402,6 +10632,12 @@
       <c r="N206" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O206">
+        <v>2</v>
+      </c>
+      <c r="P206" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
@@ -9446,6 +10682,12 @@
       <c r="N207" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O207">
+        <v>0</v>
+      </c>
+      <c r="P207" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
@@ -9490,6 +10732,12 @@
       <c r="N208" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O208">
+        <v>0</v>
+      </c>
+      <c r="P208" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
@@ -9534,6 +10782,12 @@
       <c r="N209" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O209">
+        <v>4</v>
+      </c>
+      <c r="P209" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
@@ -9578,6 +10832,12 @@
       <c r="N210" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O210">
+        <v>-2</v>
+      </c>
+      <c r="P210" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
@@ -9622,6 +10882,12 @@
       <c r="N211" t="str">
         <v>Bank</v>
       </c>
+      <c r="O211">
+        <v>2</v>
+      </c>
+      <c r="P211" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
@@ -9666,6 +10932,12 @@
       <c r="N212" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O212">
+        <v>4</v>
+      </c>
+      <c r="P212" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
@@ -9710,6 +10982,12 @@
       <c r="N213" t="str">
         <v>Bank</v>
       </c>
+      <c r="O213">
+        <v>0</v>
+      </c>
+      <c r="P213" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
@@ -9754,6 +11032,12 @@
       <c r="N214" t="str">
         <v>Bank</v>
       </c>
+      <c r="O214">
+        <v>0</v>
+      </c>
+      <c r="P214" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
@@ -9798,6 +11082,12 @@
       <c r="N215" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O215">
+        <v>8</v>
+      </c>
+      <c r="P215" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
@@ -9842,6 +11132,12 @@
       <c r="N216" t="str">
         <v>Bank</v>
       </c>
+      <c r="O216">
+        <v>-2</v>
+      </c>
+      <c r="P216" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
@@ -9886,6 +11182,12 @@
       <c r="N217" t="str">
         <v>Bank</v>
       </c>
+      <c r="O217">
+        <v>0</v>
+      </c>
+      <c r="P217" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
@@ -9930,6 +11232,12 @@
       <c r="N218" t="str">
         <v>Bank</v>
       </c>
+      <c r="O218">
+        <v>2</v>
+      </c>
+      <c r="P218" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
@@ -9974,6 +11282,12 @@
       <c r="N219" t="str">
         <v>Bank</v>
       </c>
+      <c r="O219">
+        <v>0</v>
+      </c>
+      <c r="P219" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
@@ -10018,6 +11332,12 @@
       <c r="N220" t="str">
         <v>Bank</v>
       </c>
+      <c r="O220">
+        <v>0</v>
+      </c>
+      <c r="P220" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
@@ -10062,6 +11382,12 @@
       <c r="N221" t="str">
         <v>Bank</v>
       </c>
+      <c r="O221">
+        <v>2</v>
+      </c>
+      <c r="P221" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
@@ -10106,6 +11432,12 @@
       <c r="N222" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O222">
+        <v>6</v>
+      </c>
+      <c r="P222" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
@@ -10150,6 +11482,12 @@
       <c r="N223" t="str">
         <v>Bank</v>
       </c>
+      <c r="O223">
+        <v>4</v>
+      </c>
+      <c r="P223" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
@@ -10194,6 +11532,12 @@
       <c r="N224" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O224">
+        <v>2</v>
+      </c>
+      <c r="P224" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
@@ -10238,6 +11582,12 @@
       <c r="N225" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O225">
+        <v>12</v>
+      </c>
+      <c r="P225" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
@@ -10282,6 +11632,12 @@
       <c r="N226" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O226">
+        <v>0</v>
+      </c>
+      <c r="P226" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
@@ -10326,6 +11682,12 @@
       <c r="N227" t="str">
         <v>Bank</v>
       </c>
+      <c r="O227">
+        <v>0</v>
+      </c>
+      <c r="P227" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
@@ -10370,6 +11732,12 @@
       <c r="N228" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O228">
+        <v>2</v>
+      </c>
+      <c r="P228" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
@@ -10414,6 +11782,12 @@
       <c r="N229" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O229">
+        <v>21</v>
+      </c>
+      <c r="P229" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
@@ -10458,6 +11832,12 @@
       <c r="N230" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O230">
+        <v>-2</v>
+      </c>
+      <c r="P230" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
@@ -10502,6 +11882,12 @@
       <c r="N231" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O231">
+        <v>13</v>
+      </c>
+      <c r="P231" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
@@ -10546,6 +11932,12 @@
       <c r="N232" t="str">
         <v>Bank</v>
       </c>
+      <c r="O232">
+        <v>0</v>
+      </c>
+      <c r="P232" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
@@ -10590,6 +11982,12 @@
       <c r="N233" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O233">
+        <v>2</v>
+      </c>
+      <c r="P233" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
@@ -10634,6 +12032,12 @@
       <c r="N234" t="str">
         <v>Bank</v>
       </c>
+      <c r="O234">
+        <v>0</v>
+      </c>
+      <c r="P234" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
@@ -10678,6 +12082,12 @@
       <c r="N235" t="str">
         <v>Bank</v>
       </c>
+      <c r="O235">
+        <v>0</v>
+      </c>
+      <c r="P235" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
@@ -10722,6 +12132,12 @@
       <c r="N236" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O236">
+        <v>2</v>
+      </c>
+      <c r="P236" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
@@ -10766,6 +12182,12 @@
       <c r="N237" t="str">
         <v>Bank</v>
       </c>
+      <c r="O237">
+        <v>0</v>
+      </c>
+      <c r="P237" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
@@ -10810,6 +12232,12 @@
       <c r="N238" t="str">
         <v>Bank</v>
       </c>
+      <c r="O238">
+        <v>0</v>
+      </c>
+      <c r="P238" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
@@ -10854,6 +12282,12 @@
       <c r="N239" t="str">
         <v>Bank</v>
       </c>
+      <c r="O239">
+        <v>2</v>
+      </c>
+      <c r="P239" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
@@ -10898,6 +12332,12 @@
       <c r="N240" t="str">
         <v>Bank</v>
       </c>
+      <c r="O240">
+        <v>0</v>
+      </c>
+      <c r="P240" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
@@ -10942,6 +12382,12 @@
       <c r="N241" t="str">
         <v>Bank</v>
       </c>
+      <c r="O241">
+        <v>0</v>
+      </c>
+      <c r="P241" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
@@ -10986,6 +12432,12 @@
       <c r="N242" t="str">
         <v>Startelf</v>
       </c>
+      <c r="O242">
+        <v>8</v>
+      </c>
+      <c r="P242" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
@@ -11030,10 +12482,16 @@
       <c r="N243" t="str">
         <v>Bank</v>
       </c>
+      <c r="O243">
+        <v>0</v>
+      </c>
+      <c r="P243" t="str">
+        <v>Bank</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N243"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P243"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Spieltag 7 (2026/27): Daten, Kaderseiten, Portal, Spieltagsbericht, Blick in die Geschichte, Nerdwissen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2jFkcxko3GiCvCav52Uvz
</commit_message>
<xml_diff>
--- a/saison.xlsx
+++ b/saison.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P243"/>
+  <dimension ref="A1:R243"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -448,6 +448,12 @@
       <c r="P1" t="str">
         <v>ST6 Rolle</v>
       </c>
+      <c r="Q1" t="str">
+        <v>ST7 Punkte</v>
+      </c>
+      <c r="R1" t="str">
+        <v>ST7 Rolle</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -498,6 +504,12 @@
       <c r="P2" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q2">
+        <v>8</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -548,6 +560,12 @@
       <c r="P3" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -598,6 +616,12 @@
       <c r="P4" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -648,6 +672,12 @@
       <c r="P5" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q5">
+        <v>8</v>
+      </c>
+      <c r="R5" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -698,6 +728,12 @@
       <c r="P6" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q6">
+        <v>4</v>
+      </c>
+      <c r="R6" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -748,6 +784,12 @@
       <c r="P7" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -798,6 +840,12 @@
       <c r="P8" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q8">
+        <v>2</v>
+      </c>
+      <c r="R8" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -848,6 +896,12 @@
       <c r="P9" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q9">
+        <v>2</v>
+      </c>
+      <c r="R9" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -898,6 +952,12 @@
       <c r="P10" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q10">
+        <v>15</v>
+      </c>
+      <c r="R10" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -948,6 +1008,12 @@
       <c r="P11" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -998,6 +1064,12 @@
       <c r="P12" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1048,6 +1120,12 @@
       <c r="P13" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q13">
+        <v>0</v>
+      </c>
+      <c r="R13" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1098,6 +1176,12 @@
       <c r="P14" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q14">
+        <v>0</v>
+      </c>
+      <c r="R14" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1148,6 +1232,12 @@
       <c r="P15" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q15">
+        <v>4</v>
+      </c>
+      <c r="R15" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1198,6 +1288,12 @@
       <c r="P16" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q16">
+        <v>2</v>
+      </c>
+      <c r="R16" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1248,6 +1344,12 @@
       <c r="P17" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q17">
+        <v>0</v>
+      </c>
+      <c r="R17" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1298,6 +1400,12 @@
       <c r="P18" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q18">
+        <v>2</v>
+      </c>
+      <c r="R18" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1348,6 +1456,12 @@
       <c r="P19" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q19">
+        <v>0</v>
+      </c>
+      <c r="R19" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1398,6 +1512,12 @@
       <c r="P20" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q20">
+        <v>0</v>
+      </c>
+      <c r="R20" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1448,6 +1568,12 @@
       <c r="P21" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q21">
+        <v>0</v>
+      </c>
+      <c r="R21" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1498,6 +1624,12 @@
       <c r="P22" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q22">
+        <v>0</v>
+      </c>
+      <c r="R22" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1548,6 +1680,12 @@
       <c r="P23" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q23">
+        <v>0</v>
+      </c>
+      <c r="R23" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1598,6 +1736,12 @@
       <c r="P24" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q24">
+        <v>13</v>
+      </c>
+      <c r="R24" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1648,6 +1792,12 @@
       <c r="P25" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q25">
+        <v>4</v>
+      </c>
+      <c r="R25" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1692,6 +1842,12 @@
       <c r="P26" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q26">
+        <v>0</v>
+      </c>
+      <c r="R26" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1742,6 +1898,12 @@
       <c r="P27" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q27">
+        <v>2</v>
+      </c>
+      <c r="R27" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1792,6 +1954,12 @@
       <c r="P28" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q28">
+        <v>6</v>
+      </c>
+      <c r="R28" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1842,6 +2010,12 @@
       <c r="P29" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q29">
+        <v>0</v>
+      </c>
+      <c r="R29" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1892,6 +2066,12 @@
       <c r="P30" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q30">
+        <v>0</v>
+      </c>
+      <c r="R30" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1942,6 +2122,12 @@
       <c r="P31" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q31">
+        <v>2</v>
+      </c>
+      <c r="R31" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1992,6 +2178,12 @@
       <c r="P32" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q32">
+        <v>15</v>
+      </c>
+      <c r="R32" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -2042,6 +2234,12 @@
       <c r="P33" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q33">
+        <v>6</v>
+      </c>
+      <c r="R33" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -2092,6 +2290,12 @@
       <c r="P34" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q34">
+        <v>19</v>
+      </c>
+      <c r="R34" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -2142,6 +2346,12 @@
       <c r="P35" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q35">
+        <v>0</v>
+      </c>
+      <c r="R35" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -2192,6 +2402,12 @@
       <c r="P36" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q36">
+        <v>0</v>
+      </c>
+      <c r="R36" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -2242,6 +2458,12 @@
       <c r="P37" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q37">
+        <v>0</v>
+      </c>
+      <c r="R37" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -2292,6 +2514,12 @@
       <c r="P38" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q38">
+        <v>0</v>
+      </c>
+      <c r="R38" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -2342,6 +2570,12 @@
       <c r="P39" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q39">
+        <v>0</v>
+      </c>
+      <c r="R39" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -2392,6 +2626,12 @@
       <c r="P40" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q40">
+        <v>0</v>
+      </c>
+      <c r="R40" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -2442,6 +2682,12 @@
       <c r="P41" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q41">
+        <v>0</v>
+      </c>
+      <c r="R41" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -2492,6 +2738,12 @@
       <c r="P42" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q42">
+        <v>0</v>
+      </c>
+      <c r="R42" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -2536,6 +2788,12 @@
       <c r="P43" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q43">
+        <v>0</v>
+      </c>
+      <c r="R43" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -2586,6 +2844,12 @@
       <c r="P44" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q44">
+        <v>0</v>
+      </c>
+      <c r="R44" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -2636,6 +2900,12 @@
       <c r="P45" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q45">
+        <v>2</v>
+      </c>
+      <c r="R45" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -2686,6 +2956,12 @@
       <c r="P46" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q46">
+        <v>6</v>
+      </c>
+      <c r="R46" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -2736,6 +3012,12 @@
       <c r="P47" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q47">
+        <v>10</v>
+      </c>
+      <c r="R47" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -2786,6 +3068,12 @@
       <c r="P48" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q48">
+        <v>2</v>
+      </c>
+      <c r="R48" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -2836,6 +3124,12 @@
       <c r="P49" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q49">
+        <v>0</v>
+      </c>
+      <c r="R49" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -2886,6 +3180,12 @@
       <c r="P50" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q50">
+        <v>2</v>
+      </c>
+      <c r="R50" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -2936,6 +3236,12 @@
       <c r="P51" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q51">
+        <v>0</v>
+      </c>
+      <c r="R51" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -2986,6 +3292,12 @@
       <c r="P52" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q52">
+        <v>23</v>
+      </c>
+      <c r="R52" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -3036,6 +3348,12 @@
       <c r="P53" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q53">
+        <v>4</v>
+      </c>
+      <c r="R53" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -3086,6 +3404,12 @@
       <c r="P54" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q54">
+        <v>15</v>
+      </c>
+      <c r="R54" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -3136,6 +3460,12 @@
       <c r="P55" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q55">
+        <v>0</v>
+      </c>
+      <c r="R55" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -3186,6 +3516,12 @@
       <c r="P56" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q56">
+        <v>0</v>
+      </c>
+      <c r="R56" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -3236,6 +3572,12 @@
       <c r="P57" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q57">
+        <v>0</v>
+      </c>
+      <c r="R57" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -3286,6 +3628,12 @@
       <c r="P58" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q58">
+        <v>0</v>
+      </c>
+      <c r="R58" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -3336,6 +3684,12 @@
       <c r="P59" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q59">
+        <v>0</v>
+      </c>
+      <c r="R59" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -3386,6 +3740,12 @@
       <c r="P60" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q60">
+        <v>0</v>
+      </c>
+      <c r="R60" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -3436,6 +3796,12 @@
       <c r="P61" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q61">
+        <v>0</v>
+      </c>
+      <c r="R61" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -3486,6 +3852,12 @@
       <c r="P62" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q62">
+        <v>2</v>
+      </c>
+      <c r="R62" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -3536,6 +3908,12 @@
       <c r="P63" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q63">
+        <v>0</v>
+      </c>
+      <c r="R63" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -3586,6 +3964,12 @@
       <c r="P64" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q64">
+        <v>2</v>
+      </c>
+      <c r="R64" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -3636,6 +4020,12 @@
       <c r="P65" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q65">
+        <v>4</v>
+      </c>
+      <c r="R65" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -3686,6 +4076,12 @@
       <c r="P66" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q66">
+        <v>2</v>
+      </c>
+      <c r="R66" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -3736,6 +4132,12 @@
       <c r="P67" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q67">
+        <v>0</v>
+      </c>
+      <c r="R67" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -3786,6 +4188,12 @@
       <c r="P68" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q68">
+        <v>13</v>
+      </c>
+      <c r="R68" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -3836,6 +4244,12 @@
       <c r="P69" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q69">
+        <v>8</v>
+      </c>
+      <c r="R69" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -3886,6 +4300,12 @@
       <c r="P70" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q70">
+        <v>0</v>
+      </c>
+      <c r="R70" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -3936,6 +4356,12 @@
       <c r="P71" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q71">
+        <v>0</v>
+      </c>
+      <c r="R71" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -3986,6 +4412,12 @@
       <c r="P72" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q72">
+        <v>10</v>
+      </c>
+      <c r="R72" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -4036,6 +4468,12 @@
       <c r="P73" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q73">
+        <v>2</v>
+      </c>
+      <c r="R73" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -4086,6 +4524,12 @@
       <c r="P74" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q74">
+        <v>6</v>
+      </c>
+      <c r="R74" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -4136,6 +4580,12 @@
       <c r="P75" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q75">
+        <v>4</v>
+      </c>
+      <c r="R75" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -4186,6 +4636,12 @@
       <c r="P76" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q76">
+        <v>0</v>
+      </c>
+      <c r="R76" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -4236,6 +4692,12 @@
       <c r="P77" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q77">
+        <v>4</v>
+      </c>
+      <c r="R77" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -4286,6 +4748,12 @@
       <c r="P78" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q78">
+        <v>15</v>
+      </c>
+      <c r="R78" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -4336,6 +4804,12 @@
       <c r="P79" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q79">
+        <v>0</v>
+      </c>
+      <c r="R79" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -4386,6 +4860,12 @@
       <c r="P80" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q80">
+        <v>0</v>
+      </c>
+      <c r="R80" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -4436,6 +4916,12 @@
       <c r="P81" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q81">
+        <v>0</v>
+      </c>
+      <c r="R81" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -4480,6 +4966,12 @@
       <c r="P82" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q82">
+        <v>0</v>
+      </c>
+      <c r="R82" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -4530,6 +5022,12 @@
       <c r="P83" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q83">
+        <v>4</v>
+      </c>
+      <c r="R83" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -4580,6 +5078,12 @@
       <c r="P84" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q84">
+        <v>4</v>
+      </c>
+      <c r="R84" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -4630,6 +5134,12 @@
       <c r="P85" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q85">
+        <v>2</v>
+      </c>
+      <c r="R85" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -4680,6 +5190,12 @@
       <c r="P86" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q86">
+        <v>0</v>
+      </c>
+      <c r="R86" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -4730,6 +5246,12 @@
       <c r="P87" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q87">
+        <v>0</v>
+      </c>
+      <c r="R87" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -4780,6 +5302,12 @@
       <c r="P88" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q88">
+        <v>0</v>
+      </c>
+      <c r="R88" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -4830,6 +5358,12 @@
       <c r="P89" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q89">
+        <v>0</v>
+      </c>
+      <c r="R89" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -4880,6 +5414,12 @@
       <c r="P90" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q90">
+        <v>2</v>
+      </c>
+      <c r="R90" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -4930,6 +5470,12 @@
       <c r="P91" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q91">
+        <v>2</v>
+      </c>
+      <c r="R91" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -4980,6 +5526,12 @@
       <c r="P92" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q92">
+        <v>10</v>
+      </c>
+      <c r="R92" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -5030,6 +5582,12 @@
       <c r="P93" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q93">
+        <v>2</v>
+      </c>
+      <c r="R93" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -5080,6 +5638,12 @@
       <c r="P94" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q94">
+        <v>0</v>
+      </c>
+      <c r="R94" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -5130,6 +5694,12 @@
       <c r="P95" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q95">
+        <v>0</v>
+      </c>
+      <c r="R95" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -5180,6 +5750,12 @@
       <c r="P96" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q96">
+        <v>0</v>
+      </c>
+      <c r="R96" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -5230,6 +5806,12 @@
       <c r="P97" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q97">
+        <v>4</v>
+      </c>
+      <c r="R97" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -5280,6 +5862,12 @@
       <c r="P98" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q98">
+        <v>-4</v>
+      </c>
+      <c r="R98" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -5330,6 +5918,12 @@
       <c r="P99" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q99">
+        <v>0</v>
+      </c>
+      <c r="R99" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -5380,6 +5974,12 @@
       <c r="P100" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q100">
+        <v>4</v>
+      </c>
+      <c r="R100" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -5430,6 +6030,12 @@
       <c r="P101" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q101">
+        <v>0</v>
+      </c>
+      <c r="R101" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -5480,6 +6086,12 @@
       <c r="P102" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q102">
+        <v>0</v>
+      </c>
+      <c r="R102" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -5530,6 +6142,12 @@
       <c r="P103" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q103">
+        <v>0</v>
+      </c>
+      <c r="R103" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -5574,6 +6192,12 @@
       <c r="P104" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q104">
+        <v>0</v>
+      </c>
+      <c r="R104" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -5624,6 +6248,12 @@
       <c r="P105" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q105">
+        <v>0</v>
+      </c>
+      <c r="R105" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -5674,6 +6304,12 @@
       <c r="P106" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q106">
+        <v>4</v>
+      </c>
+      <c r="R106" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -5718,6 +6354,12 @@
       <c r="P107" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q107">
+        <v>0</v>
+      </c>
+      <c r="R107" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -5768,6 +6410,12 @@
       <c r="P108" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q108">
+        <v>2</v>
+      </c>
+      <c r="R108" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -5818,6 +6466,12 @@
       <c r="P109" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q109">
+        <v>2</v>
+      </c>
+      <c r="R109" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -5868,6 +6522,12 @@
       <c r="P110" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q110">
+        <v>0</v>
+      </c>
+      <c r="R110" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -5912,6 +6572,12 @@
       <c r="P111" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q111">
+        <v>0</v>
+      </c>
+      <c r="R111" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -5962,6 +6628,12 @@
       <c r="P112" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q112">
+        <v>4</v>
+      </c>
+      <c r="R112" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -6012,6 +6684,12 @@
       <c r="P113" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q113">
+        <v>4</v>
+      </c>
+      <c r="R113" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -6062,6 +6740,12 @@
       <c r="P114" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q114">
+        <v>0</v>
+      </c>
+      <c r="R114" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -6112,6 +6796,12 @@
       <c r="P115" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q115">
+        <v>0</v>
+      </c>
+      <c r="R115" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -6162,6 +6852,12 @@
       <c r="P116" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q116">
+        <v>0</v>
+      </c>
+      <c r="R116" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -6212,6 +6908,12 @@
       <c r="P117" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q117">
+        <v>2</v>
+      </c>
+      <c r="R117" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -6262,6 +6964,12 @@
       <c r="P118" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q118">
+        <v>2</v>
+      </c>
+      <c r="R118" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -6312,6 +7020,12 @@
       <c r="P119" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q119">
+        <v>0</v>
+      </c>
+      <c r="R119" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -6362,6 +7076,12 @@
       <c r="P120" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q120">
+        <v>12</v>
+      </c>
+      <c r="R120" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -6412,6 +7132,12 @@
       <c r="P121" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q121">
+        <v>0</v>
+      </c>
+      <c r="R121" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -6462,6 +7188,12 @@
       <c r="P122" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q122">
+        <v>6</v>
+      </c>
+      <c r="R122" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -6512,6 +7244,12 @@
       <c r="P123" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q123">
+        <v>0</v>
+      </c>
+      <c r="R123" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -6562,6 +7300,12 @@
       <c r="P124" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q124">
+        <v>0</v>
+      </c>
+      <c r="R124" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -6612,6 +7356,12 @@
       <c r="P125" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q125">
+        <v>0</v>
+      </c>
+      <c r="R125" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -6656,6 +7406,12 @@
       <c r="P126" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q126">
+        <v>0</v>
+      </c>
+      <c r="R126" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -6706,6 +7462,12 @@
       <c r="P127" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q127">
+        <v>0</v>
+      </c>
+      <c r="R127" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -6756,6 +7518,12 @@
       <c r="P128" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q128">
+        <v>0</v>
+      </c>
+      <c r="R128" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
@@ -6806,6 +7574,12 @@
       <c r="P129" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q129">
+        <v>2</v>
+      </c>
+      <c r="R129" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
@@ -6856,6 +7630,12 @@
       <c r="P130" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q130">
+        <v>0</v>
+      </c>
+      <c r="R130" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
@@ -6900,6 +7680,12 @@
       <c r="P131" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q131">
+        <v>0</v>
+      </c>
+      <c r="R131" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
@@ -6950,6 +7736,12 @@
       <c r="P132" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q132">
+        <v>2</v>
+      </c>
+      <c r="R132" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
@@ -7000,6 +7792,12 @@
       <c r="P133" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q133">
+        <v>4</v>
+      </c>
+      <c r="R133" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -7050,6 +7848,12 @@
       <c r="P134" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q134">
+        <v>0</v>
+      </c>
+      <c r="R134" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
@@ -7100,6 +7904,12 @@
       <c r="P135" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q135">
+        <v>0</v>
+      </c>
+      <c r="R135" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
@@ -7150,6 +7960,12 @@
       <c r="P136" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q136">
+        <v>0</v>
+      </c>
+      <c r="R136" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
@@ -7200,6 +8016,12 @@
       <c r="P137" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q137">
+        <v>10</v>
+      </c>
+      <c r="R137" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
@@ -7250,6 +8072,12 @@
       <c r="P138" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q138">
+        <v>13</v>
+      </c>
+      <c r="R138" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
@@ -7300,6 +8128,12 @@
       <c r="P139" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q139">
+        <v>6</v>
+      </c>
+      <c r="R139" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
@@ -7350,6 +8184,12 @@
       <c r="P140" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q140">
+        <v>0</v>
+      </c>
+      <c r="R140" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
@@ -7400,6 +8240,12 @@
       <c r="P141" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q141">
+        <v>23</v>
+      </c>
+      <c r="R141" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
@@ -7450,6 +8296,12 @@
       <c r="P142" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q142">
+        <v>2</v>
+      </c>
+      <c r="R142" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
@@ -7500,6 +8352,12 @@
       <c r="P143" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q143">
+        <v>6</v>
+      </c>
+      <c r="R143" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
@@ -7550,6 +8408,12 @@
       <c r="P144" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q144">
+        <v>0</v>
+      </c>
+      <c r="R144" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
@@ -7600,6 +8464,12 @@
       <c r="P145" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q145">
+        <v>6</v>
+      </c>
+      <c r="R145" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
@@ -7650,6 +8520,12 @@
       <c r="P146" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q146">
+        <v>0</v>
+      </c>
+      <c r="R146" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
@@ -7700,6 +8576,12 @@
       <c r="P147" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q147">
+        <v>0</v>
+      </c>
+      <c r="R147" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
@@ -7750,6 +8632,12 @@
       <c r="P148" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q148">
+        <v>4</v>
+      </c>
+      <c r="R148" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
@@ -7800,6 +8688,12 @@
       <c r="P149" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q149">
+        <v>0</v>
+      </c>
+      <c r="R149" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
@@ -7850,6 +8744,12 @@
       <c r="P150" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q150">
+        <v>0</v>
+      </c>
+      <c r="R150" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
@@ -7900,6 +8800,12 @@
       <c r="P151" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q151">
+        <v>0</v>
+      </c>
+      <c r="R151" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
@@ -7950,6 +8856,12 @@
       <c r="P152" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q152">
+        <v>0</v>
+      </c>
+      <c r="R152" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
@@ -8000,6 +8912,12 @@
       <c r="P153" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q153">
+        <v>2</v>
+      </c>
+      <c r="R153" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
@@ -8050,6 +8968,12 @@
       <c r="P154" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q154">
+        <v>0</v>
+      </c>
+      <c r="R154" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
@@ -8100,6 +9024,12 @@
       <c r="P155" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q155">
+        <v>0</v>
+      </c>
+      <c r="R155" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
@@ -8150,6 +9080,12 @@
       <c r="P156" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q156">
+        <v>4</v>
+      </c>
+      <c r="R156" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
@@ -8200,6 +9136,12 @@
       <c r="P157" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q157">
+        <v>4</v>
+      </c>
+      <c r="R157" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
@@ -8250,6 +9192,12 @@
       <c r="P158" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q158">
+        <v>8</v>
+      </c>
+      <c r="R158" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
@@ -8300,6 +9248,12 @@
       <c r="P159" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q159">
+        <v>0</v>
+      </c>
+      <c r="R159" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
@@ -8350,6 +9304,12 @@
       <c r="P160" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q160">
+        <v>0</v>
+      </c>
+      <c r="R160" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
@@ -8400,6 +9360,12 @@
       <c r="P161" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q161">
+        <v>0</v>
+      </c>
+      <c r="R161" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
@@ -8450,6 +9416,12 @@
       <c r="P162" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q162">
+        <v>10</v>
+      </c>
+      <c r="R162" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
@@ -8500,6 +9472,12 @@
       <c r="P163" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q163">
+        <v>6</v>
+      </c>
+      <c r="R163" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
@@ -8550,6 +9528,12 @@
       <c r="P164" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q164">
+        <v>0</v>
+      </c>
+      <c r="R164" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
@@ -8600,6 +9584,12 @@
       <c r="P165" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q165">
+        <v>19</v>
+      </c>
+      <c r="R165" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
@@ -8650,6 +9640,12 @@
       <c r="P166" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q166">
+        <v>0</v>
+      </c>
+      <c r="R166" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
@@ -8700,6 +9696,12 @@
       <c r="P167" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q167">
+        <v>0</v>
+      </c>
+      <c r="R167" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
@@ -8750,6 +9752,12 @@
       <c r="P168" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q168">
+        <v>0</v>
+      </c>
+      <c r="R168" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
@@ -8800,6 +9808,12 @@
       <c r="P169" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q169">
+        <v>0</v>
+      </c>
+      <c r="R169" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
@@ -8850,6 +9864,12 @@
       <c r="P170" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q170">
+        <v>4</v>
+      </c>
+      <c r="R170" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
@@ -8900,6 +9920,12 @@
       <c r="P171" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q171">
+        <v>0</v>
+      </c>
+      <c r="R171" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
@@ -8950,6 +9976,12 @@
       <c r="P172" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q172">
+        <v>0</v>
+      </c>
+      <c r="R172" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
@@ -9000,6 +10032,12 @@
       <c r="P173" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q173">
+        <v>0</v>
+      </c>
+      <c r="R173" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
@@ -9050,6 +10088,12 @@
       <c r="P174" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q174">
+        <v>0</v>
+      </c>
+      <c r="R174" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
@@ -9100,6 +10144,12 @@
       <c r="P175" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q175">
+        <v>0</v>
+      </c>
+      <c r="R175" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
@@ -9150,6 +10200,12 @@
       <c r="P176" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q176">
+        <v>6</v>
+      </c>
+      <c r="R176" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
@@ -9200,6 +10256,12 @@
       <c r="P177" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q177">
+        <v>0</v>
+      </c>
+      <c r="R177" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
@@ -9250,6 +10312,12 @@
       <c r="P178" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q178">
+        <v>0</v>
+      </c>
+      <c r="R178" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
@@ -9300,6 +10368,12 @@
       <c r="P179" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q179">
+        <v>4</v>
+      </c>
+      <c r="R179" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
@@ -9350,6 +10424,12 @@
       <c r="P180" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q180">
+        <v>0</v>
+      </c>
+      <c r="R180" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
@@ -9400,6 +10480,12 @@
       <c r="P181" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q181">
+        <v>0</v>
+      </c>
+      <c r="R181" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
@@ -9450,6 +10536,12 @@
       <c r="P182" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q182">
+        <v>6</v>
+      </c>
+      <c r="R182" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
@@ -9500,6 +10592,12 @@
       <c r="P183" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q183">
+        <v>2</v>
+      </c>
+      <c r="R183" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
@@ -9550,6 +10648,12 @@
       <c r="P184" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q184">
+        <v>2</v>
+      </c>
+      <c r="R184" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
@@ -9600,6 +10704,12 @@
       <c r="P185" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q185">
+        <v>10</v>
+      </c>
+      <c r="R185" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
@@ -9650,6 +10760,12 @@
       <c r="P186" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q186">
+        <v>-4</v>
+      </c>
+      <c r="R186" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
@@ -9700,6 +10816,12 @@
       <c r="P187" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q187">
+        <v>0</v>
+      </c>
+      <c r="R187" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
@@ -9750,6 +10872,12 @@
       <c r="P188" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q188">
+        <v>2</v>
+      </c>
+      <c r="R188" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
@@ -9800,6 +10928,12 @@
       <c r="P189" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q189">
+        <v>0</v>
+      </c>
+      <c r="R189" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
@@ -9850,6 +10984,12 @@
       <c r="P190" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q190">
+        <v>0</v>
+      </c>
+      <c r="R190" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
@@ -9900,6 +11040,12 @@
       <c r="P191" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q191">
+        <v>0</v>
+      </c>
+      <c r="R191" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
@@ -9950,6 +11096,12 @@
       <c r="P192" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q192">
+        <v>0</v>
+      </c>
+      <c r="R192" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
@@ -9994,6 +11146,12 @@
       <c r="P193" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q193">
+        <v>0</v>
+      </c>
+      <c r="R193" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
@@ -10044,6 +11202,12 @@
       <c r="P194" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q194">
+        <v>0</v>
+      </c>
+      <c r="R194" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
@@ -10094,6 +11258,12 @@
       <c r="P195" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q195">
+        <v>0</v>
+      </c>
+      <c r="R195" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
@@ -10144,6 +11314,12 @@
       <c r="P196" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q196">
+        <v>0</v>
+      </c>
+      <c r="R196" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
@@ -10194,6 +11370,12 @@
       <c r="P197" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q197">
+        <v>4</v>
+      </c>
+      <c r="R197" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
@@ -10238,6 +11420,12 @@
       <c r="P198" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q198">
+        <v>0</v>
+      </c>
+      <c r="R198" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
@@ -10288,6 +11476,12 @@
       <c r="P199" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q199">
+        <v>0</v>
+      </c>
+      <c r="R199" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
@@ -10338,6 +11532,12 @@
       <c r="P200" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q200">
+        <v>0</v>
+      </c>
+      <c r="R200" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
@@ -10388,6 +11588,12 @@
       <c r="P201" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q201">
+        <v>13</v>
+      </c>
+      <c r="R201" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
@@ -10438,6 +11644,12 @@
       <c r="P202" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q202">
+        <v>2</v>
+      </c>
+      <c r="R202" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
@@ -10488,6 +11700,12 @@
       <c r="P203" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q203">
+        <v>0</v>
+      </c>
+      <c r="R203" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
@@ -10538,6 +11756,12 @@
       <c r="P204" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q204">
+        <v>2</v>
+      </c>
+      <c r="R204" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
@@ -10588,6 +11812,12 @@
       <c r="P205" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q205">
+        <v>2</v>
+      </c>
+      <c r="R205" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
@@ -10638,6 +11868,12 @@
       <c r="P206" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q206">
+        <v>2</v>
+      </c>
+      <c r="R206" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
@@ -10688,6 +11924,12 @@
       <c r="P207" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q207">
+        <v>2</v>
+      </c>
+      <c r="R207" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
@@ -10738,6 +11980,12 @@
       <c r="P208" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q208">
+        <v>6</v>
+      </c>
+      <c r="R208" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
@@ -10788,6 +12036,12 @@
       <c r="P209" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q209">
+        <v>4</v>
+      </c>
+      <c r="R209" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
@@ -10838,6 +12092,12 @@
       <c r="P210" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q210">
+        <v>0</v>
+      </c>
+      <c r="R210" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
@@ -10888,6 +12148,12 @@
       <c r="P211" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q211">
+        <v>2</v>
+      </c>
+      <c r="R211" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
@@ -10938,6 +12204,12 @@
       <c r="P212" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q212">
+        <v>0</v>
+      </c>
+      <c r="R212" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
@@ -10988,6 +12260,12 @@
       <c r="P213" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q213">
+        <v>4</v>
+      </c>
+      <c r="R213" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
@@ -11038,6 +12316,12 @@
       <c r="P214" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q214">
+        <v>0</v>
+      </c>
+      <c r="R214" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
@@ -11088,6 +12372,12 @@
       <c r="P215" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q215">
+        <v>0</v>
+      </c>
+      <c r="R215" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
@@ -11138,6 +12428,12 @@
       <c r="P216" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q216">
+        <v>0</v>
+      </c>
+      <c r="R216" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
@@ -11188,6 +12484,12 @@
       <c r="P217" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q217">
+        <v>0</v>
+      </c>
+      <c r="R217" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
@@ -11238,6 +12540,12 @@
       <c r="P218" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q218">
+        <v>0</v>
+      </c>
+      <c r="R218" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
@@ -11288,6 +12596,12 @@
       <c r="P219" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q219">
+        <v>2</v>
+      </c>
+      <c r="R219" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
@@ -11338,6 +12652,12 @@
       <c r="P220" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q220">
+        <v>0</v>
+      </c>
+      <c r="R220" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
@@ -11388,6 +12708,12 @@
       <c r="P221" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q221">
+        <v>2</v>
+      </c>
+      <c r="R221" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
@@ -11438,6 +12764,12 @@
       <c r="P222" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q222">
+        <v>0</v>
+      </c>
+      <c r="R222" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
@@ -11488,6 +12820,12 @@
       <c r="P223" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q223">
+        <v>4</v>
+      </c>
+      <c r="R223" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
@@ -11538,6 +12876,12 @@
       <c r="P224" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q224">
+        <v>8</v>
+      </c>
+      <c r="R224" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
@@ -11588,6 +12932,12 @@
       <c r="P225" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q225">
+        <v>10</v>
+      </c>
+      <c r="R225" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
@@ -11638,6 +12988,12 @@
       <c r="P226" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q226">
+        <v>2</v>
+      </c>
+      <c r="R226" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
@@ -11688,6 +13044,12 @@
       <c r="P227" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q227">
+        <v>0</v>
+      </c>
+      <c r="R227" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
@@ -11738,6 +13100,12 @@
       <c r="P228" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q228">
+        <v>2</v>
+      </c>
+      <c r="R228" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
@@ -11788,6 +13156,12 @@
       <c r="P229" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q229">
+        <v>2</v>
+      </c>
+      <c r="R229" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
@@ -11838,6 +13212,12 @@
       <c r="P230" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q230">
+        <v>0</v>
+      </c>
+      <c r="R230" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
@@ -11888,6 +13268,12 @@
       <c r="P231" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q231">
+        <v>0</v>
+      </c>
+      <c r="R231" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
@@ -11938,6 +13324,12 @@
       <c r="P232" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q232">
+        <v>0</v>
+      </c>
+      <c r="R232" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
@@ -11988,6 +13380,12 @@
       <c r="P233" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q233">
+        <v>4</v>
+      </c>
+      <c r="R233" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
@@ -12038,6 +13436,12 @@
       <c r="P234" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q234">
+        <v>4</v>
+      </c>
+      <c r="R234" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
@@ -12088,6 +13492,12 @@
       <c r="P235" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q235">
+        <v>0</v>
+      </c>
+      <c r="R235" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
@@ -12138,6 +13548,12 @@
       <c r="P236" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q236">
+        <v>2</v>
+      </c>
+      <c r="R236" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
@@ -12188,6 +13604,12 @@
       <c r="P237" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q237">
+        <v>0</v>
+      </c>
+      <c r="R237" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
@@ -12238,6 +13660,12 @@
       <c r="P238" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q238">
+        <v>0</v>
+      </c>
+      <c r="R238" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
@@ -12288,6 +13716,12 @@
       <c r="P239" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q239">
+        <v>0</v>
+      </c>
+      <c r="R239" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
@@ -12338,6 +13772,12 @@
       <c r="P240" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q240">
+        <v>0</v>
+      </c>
+      <c r="R240" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
@@ -12388,6 +13828,12 @@
       <c r="P241" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q241">
+        <v>0</v>
+      </c>
+      <c r="R241" t="str">
+        <v>Bank</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
@@ -12438,6 +13884,12 @@
       <c r="P242" t="str">
         <v>Startelf</v>
       </c>
+      <c r="Q242">
+        <v>0</v>
+      </c>
+      <c r="R242" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
@@ -12488,10 +13940,16 @@
       <c r="P243" t="str">
         <v>Bank</v>
       </c>
+      <c r="Q243">
+        <v>2</v>
+      </c>
+      <c r="R243" t="str">
+        <v>Startelf</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P243"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R243"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>